<commit_message>
Porcentaje aciertos y erorres
</commit_message>
<xml_diff>
--- a/datosNivelesMedias.xlsx
+++ b/datosNivelesMedias.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\hlocal\C_TFG\Datos\Mision Colombia-20260209T150018Z-3-001\jsonToCsv_TFG\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{126458BE-AB9C-435A-99A4-4B4CEE6FB0D9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1EE89827-D12E-424C-8AB3-B11868D2B383}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -56,7 +56,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="479" uniqueCount="342">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="905" uniqueCount="428">
   <si>
     <t>ID</t>
   </si>
@@ -1082,13 +1082,271 @@
   </si>
   <si>
     <t>15:42:14.394</t>
+  </si>
+  <si>
+    <t>% Aciertos</t>
+  </si>
+  <si>
+    <t>% Mal</t>
+  </si>
+  <si>
+    <t>78.57142857142857</t>
+  </si>
+  <si>
+    <t>21.42857142857143</t>
+  </si>
+  <si>
+    <t>100.0</t>
+  </si>
+  <si>
+    <t>0.0</t>
+  </si>
+  <si>
+    <t>77.77777777777777</t>
+  </si>
+  <si>
+    <t>22.22222222222223</t>
+  </si>
+  <si>
+    <t>0 planificado</t>
+  </si>
+  <si>
+    <t>80.0</t>
+  </si>
+  <si>
+    <t>20.0</t>
+  </si>
+  <si>
+    <t>90.0</t>
+  </si>
+  <si>
+    <t>10.0</t>
+  </si>
+  <si>
+    <t>83.33333333333333</t>
+  </si>
+  <si>
+    <t>16.66666666666667</t>
+  </si>
+  <si>
+    <t>75.0</t>
+  </si>
+  <si>
+    <t>25.0</t>
+  </si>
+  <si>
+    <t>85.71428571428571</t>
+  </si>
+  <si>
+    <t>14.285714285714292</t>
+  </si>
+  <si>
+    <t>50.0</t>
+  </si>
+  <si>
+    <t>94.44444444444444</t>
+  </si>
+  <si>
+    <t>5.555555555555557</t>
+  </si>
+  <si>
+    <t>88.88888888888889</t>
+  </si>
+  <si>
+    <t>11.111111111111114</t>
+  </si>
+  <si>
+    <t>76.47058823529412</t>
+  </si>
+  <si>
+    <t>23.529411764705884</t>
+  </si>
+  <si>
+    <t>60.0</t>
+  </si>
+  <si>
+    <t>40.0</t>
+  </si>
+  <si>
+    <t>87.5</t>
+  </si>
+  <si>
+    <t>12.5</t>
+  </si>
+  <si>
+    <t>76.92307692307692</t>
+  </si>
+  <si>
+    <t>23.07692307692308</t>
+  </si>
+  <si>
+    <t>90.47619047619048</t>
+  </si>
+  <si>
+    <t>9.523809523809518</t>
+  </si>
+  <si>
+    <t>86.66666666666667</t>
+  </si>
+  <si>
+    <t>13.333333333333329</t>
+  </si>
+  <si>
+    <t>88.46153846153847</t>
+  </si>
+  <si>
+    <t>11.538461538461533</t>
+  </si>
+  <si>
+    <t>72.72727272727273</t>
+  </si>
+  <si>
+    <t>27.272727272727266</t>
+  </si>
+  <si>
+    <t>93.93939393939394</t>
+  </si>
+  <si>
+    <t>6.060606060606062</t>
+  </si>
+  <si>
+    <t>73.6842105263158</t>
+  </si>
+  <si>
+    <t>26.315789473684205</t>
+  </si>
+  <si>
+    <t>90.9090909090909</t>
+  </si>
+  <si>
+    <t>9.090909090909093</t>
+  </si>
+  <si>
+    <t>79.16666666666667</t>
+  </si>
+  <si>
+    <t>20.83333333333333</t>
+  </si>
+  <si>
+    <t>71.42857142857143</t>
+  </si>
+  <si>
+    <t>28.57142857142857</t>
+  </si>
+  <si>
+    <t>66.66666666666667</t>
+  </si>
+  <si>
+    <t>33.33333333333333</t>
+  </si>
+  <si>
+    <t>54.54545454545455</t>
+  </si>
+  <si>
+    <t>45.45454545454545</t>
+  </si>
+  <si>
+    <t>86.36363636363636</t>
+  </si>
+  <si>
+    <t>13.63636363636364</t>
+  </si>
+  <si>
+    <t>72.5</t>
+  </si>
+  <si>
+    <t>27.5</t>
+  </si>
+  <si>
+    <t>81.25</t>
+  </si>
+  <si>
+    <t>18.75</t>
+  </si>
+  <si>
+    <t>92.3076923076923</t>
+  </si>
+  <si>
+    <t>7.692307692307693</t>
+  </si>
+  <si>
+    <t>93.33333333333333</t>
+  </si>
+  <si>
+    <t>6.666666666666671</t>
+  </si>
+  <si>
+    <t>35.714285714285715</t>
+  </si>
+  <si>
+    <t>64.28571428571428</t>
+  </si>
+  <si>
+    <t>61.111111111111114</t>
+  </si>
+  <si>
+    <t>38.888888888888886</t>
+  </si>
+  <si>
+    <t>69.56521739130434</t>
+  </si>
+  <si>
+    <t>30.434782608695656</t>
+  </si>
+  <si>
+    <t>93.54838709677419</t>
+  </si>
+  <si>
+    <t>6.451612903225808</t>
+  </si>
+  <si>
+    <t>51.61290322580645</t>
+  </si>
+  <si>
+    <t>48.38709677419355</t>
+  </si>
+  <si>
+    <t>88.23529411764706</t>
+  </si>
+  <si>
+    <t>11.764705882352942</t>
+  </si>
+  <si>
+    <t>75.86206896551724</t>
+  </si>
+  <si>
+    <t>24.13793103448276</t>
+  </si>
+  <si>
+    <t>76.0</t>
+  </si>
+  <si>
+    <t>24.0</t>
+  </si>
+  <si>
+    <t>93.75</t>
+  </si>
+  <si>
+    <t>6.25</t>
+  </si>
+  <si>
+    <t>64.28571428571429</t>
+  </si>
+  <si>
+    <t>35.71428571428571</t>
+  </si>
+  <si>
+    <t>82.3529411764706</t>
+  </si>
+  <si>
+    <t>17.647058823529406</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1100,6 +1358,14 @@
       <b/>
       <sz val="11"/>
       <name val="Calibri"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
@@ -1135,11 +1401,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1201,9 +1468,9 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{E64F33C9-0D6E-4466-A947-979A97EAB1CA}" name="dataNiveles" displayName="dataNiveles" ref="A1:U213" totalsRowShown="0" headerRowDxfId="2" headerRowBorderDxfId="1" tableBorderDxfId="0">
-  <autoFilter ref="A1:U213" xr:uid="{E64F33C9-0D6E-4466-A947-979A97EAB1CA}"/>
-  <tableColumns count="21">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{E64F33C9-0D6E-4466-A947-979A97EAB1CA}" name="dataNiveles" displayName="dataNiveles" ref="A1:W213" totalsRowShown="0" headerRowDxfId="2" headerRowBorderDxfId="1" tableBorderDxfId="0">
+  <autoFilter ref="A1:W213" xr:uid="{E64F33C9-0D6E-4466-A947-979A97EAB1CA}"/>
+  <tableColumns count="23">
     <tableColumn id="1" xr3:uid="{0DF82F0A-802F-4E90-B194-6AF1DDF506EA}" name="ID"/>
     <tableColumn id="2" xr3:uid="{88AE4975-BA64-4005-B9D1-961ED97FEF8E}" name="Sesion"/>
     <tableColumn id="3" xr3:uid="{AD94318C-D82A-4BB8-8133-C3C07DC11584}" name="Nivel"/>
@@ -1225,6 +1492,8 @@
     <tableColumn id="19" xr3:uid="{E007CE99-01AE-4726-9425-A3644589FE2C}" name="Paradas realizadas"/>
     <tableColumn id="20" xr3:uid="{394DC09F-0F38-4A14-A268-E7C08E60C741}" name="Errores parada por tiempo excedido"/>
     <tableColumn id="21" xr3:uid="{9945298E-8DC5-4CAD-A4E8-711FB82860B0}" name="Num errores por tiempo excedido"/>
+    <tableColumn id="22" xr3:uid="{E9CFE53D-3AD7-431C-BCDA-B2435D56D455}" name="% Aciertos"/>
+    <tableColumn id="23" xr3:uid="{04189E72-7631-4376-A357-3F6F8DE60B31}" name="% Mal"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1515,7 +1784,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:U213"/>
+  <dimension ref="A1:X213"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="4" max="4" width="14.33203125" customWidth="1"/>
@@ -1535,9 +1804,10 @@
     <col min="19" max="19" width="18.21875" customWidth="1"/>
     <col min="20" max="20" width="32.88671875" customWidth="1"/>
     <col min="21" max="21" width="31.109375" customWidth="1"/>
+    <col min="22" max="23" width="18.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:21" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1601,8 +1871,14 @@
       <c r="U1" s="1" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="2" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="V1" s="1" t="s">
+        <v>342</v>
+      </c>
+      <c r="W1" s="1" t="s">
+        <v>343</v>
+      </c>
+    </row>
+    <row r="2" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A2">
         <v>10</v>
       </c>
@@ -1666,8 +1942,14 @@
       <c r="U2">
         <v>0</v>
       </c>
-    </row>
-    <row r="3" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="V2" t="s">
+        <v>344</v>
+      </c>
+      <c r="W2" t="s">
+        <v>345</v>
+      </c>
+    </row>
+    <row r="3" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A3">
         <v>10</v>
       </c>
@@ -1731,8 +2013,14 @@
       <c r="U3">
         <v>0</v>
       </c>
-    </row>
-    <row r="4" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="V3" t="s">
+        <v>346</v>
+      </c>
+      <c r="W3" t="s">
+        <v>347</v>
+      </c>
+    </row>
+    <row r="4" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A4">
         <v>10</v>
       </c>
@@ -1796,8 +2084,14 @@
       <c r="U4">
         <v>1</v>
       </c>
-    </row>
-    <row r="5" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="V4" t="s">
+        <v>346</v>
+      </c>
+      <c r="W4" t="s">
+        <v>347</v>
+      </c>
+    </row>
+    <row r="5" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A5">
         <v>10</v>
       </c>
@@ -1861,8 +2155,14 @@
       <c r="U5">
         <v>1</v>
       </c>
-    </row>
-    <row r="6" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="V5" t="s">
+        <v>348</v>
+      </c>
+      <c r="W5" t="s">
+        <v>349</v>
+      </c>
+    </row>
+    <row r="6" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A6">
         <v>10</v>
       </c>
@@ -1926,8 +2226,14 @@
       <c r="U6">
         <v>0</v>
       </c>
-    </row>
-    <row r="7" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="V6" t="s">
+        <v>350</v>
+      </c>
+      <c r="W6" t="s">
+        <v>350</v>
+      </c>
+    </row>
+    <row r="7" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A7">
         <v>11</v>
       </c>
@@ -1991,8 +2297,14 @@
       <c r="U7">
         <v>0</v>
       </c>
-    </row>
-    <row r="8" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="V7" t="s">
+        <v>351</v>
+      </c>
+      <c r="W7" t="s">
+        <v>352</v>
+      </c>
+    </row>
+    <row r="8" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A8">
         <v>11</v>
       </c>
@@ -2056,8 +2368,14 @@
       <c r="U8">
         <v>1</v>
       </c>
-    </row>
-    <row r="9" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="V8" t="s">
+        <v>353</v>
+      </c>
+      <c r="W8" t="s">
+        <v>354</v>
+      </c>
+    </row>
+    <row r="9" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A9">
         <v>11</v>
       </c>
@@ -2121,8 +2439,15 @@
       <c r="U9">
         <v>0</v>
       </c>
-    </row>
-    <row r="10" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="V9" t="s">
+        <v>355</v>
+      </c>
+      <c r="W9" t="s">
+        <v>356</v>
+      </c>
+      <c r="X9" s="2"/>
+    </row>
+    <row r="10" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A10">
         <v>11</v>
       </c>
@@ -2186,8 +2511,14 @@
       <c r="U10">
         <v>0</v>
       </c>
-    </row>
-    <row r="11" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="V10" t="s">
+        <v>348</v>
+      </c>
+      <c r="W10" t="s">
+        <v>349</v>
+      </c>
+    </row>
+    <row r="11" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A11">
         <v>11</v>
       </c>
@@ -2251,8 +2582,14 @@
       <c r="U11">
         <v>0</v>
       </c>
-    </row>
-    <row r="12" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="V11" t="s">
+        <v>346</v>
+      </c>
+      <c r="W11" t="s">
+        <v>347</v>
+      </c>
+    </row>
+    <row r="12" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A12">
         <v>11</v>
       </c>
@@ -2316,8 +2653,14 @@
       <c r="U12">
         <v>0</v>
       </c>
-    </row>
-    <row r="13" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="V12" t="s">
+        <v>355</v>
+      </c>
+      <c r="W12" t="s">
+        <v>356</v>
+      </c>
+    </row>
+    <row r="13" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A13">
         <v>11</v>
       </c>
@@ -2381,8 +2724,14 @@
       <c r="U13">
         <v>0</v>
       </c>
-    </row>
-    <row r="14" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="V13" t="s">
+        <v>350</v>
+      </c>
+      <c r="W13" t="s">
+        <v>350</v>
+      </c>
+    </row>
+    <row r="14" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A14">
         <v>13</v>
       </c>
@@ -2446,8 +2795,14 @@
       <c r="U14">
         <v>0</v>
       </c>
-    </row>
-    <row r="15" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="V14" t="s">
+        <v>346</v>
+      </c>
+      <c r="W14" t="s">
+        <v>347</v>
+      </c>
+    </row>
+    <row r="15" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A15">
         <v>13</v>
       </c>
@@ -2511,8 +2866,14 @@
       <c r="U15">
         <v>0</v>
       </c>
-    </row>
-    <row r="16" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="V15" t="s">
+        <v>346</v>
+      </c>
+      <c r="W15" t="s">
+        <v>347</v>
+      </c>
+    </row>
+    <row r="16" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A16">
         <v>13</v>
       </c>
@@ -2576,8 +2937,14 @@
       <c r="U16">
         <v>1</v>
       </c>
-    </row>
-    <row r="17" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="V16" t="s">
+        <v>357</v>
+      </c>
+      <c r="W16" t="s">
+        <v>358</v>
+      </c>
+    </row>
+    <row r="17" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A17">
         <v>13</v>
       </c>
@@ -2641,8 +3008,14 @@
       <c r="U17">
         <v>0</v>
       </c>
-    </row>
-    <row r="18" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="V17" t="s">
+        <v>346</v>
+      </c>
+      <c r="W17" t="s">
+        <v>347</v>
+      </c>
+    </row>
+    <row r="18" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A18">
         <v>13</v>
       </c>
@@ -2706,8 +3079,14 @@
       <c r="U18">
         <v>1</v>
       </c>
-    </row>
-    <row r="19" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="V18" t="s">
+        <v>346</v>
+      </c>
+      <c r="W18" t="s">
+        <v>347</v>
+      </c>
+    </row>
+    <row r="19" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A19">
         <v>13</v>
       </c>
@@ -2771,8 +3150,14 @@
       <c r="U19">
         <v>0</v>
       </c>
-    </row>
-    <row r="20" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="V19" t="s">
+        <v>359</v>
+      </c>
+      <c r="W19" t="s">
+        <v>360</v>
+      </c>
+    </row>
+    <row r="20" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A20">
         <v>15</v>
       </c>
@@ -2836,8 +3221,14 @@
       <c r="U20">
         <v>0</v>
       </c>
-    </row>
-    <row r="21" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="V20" t="s">
+        <v>350</v>
+      </c>
+      <c r="W20" t="s">
+        <v>350</v>
+      </c>
+    </row>
+    <row r="21" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A21">
         <v>15</v>
       </c>
@@ -2901,8 +3292,14 @@
       <c r="U21">
         <v>2</v>
       </c>
-    </row>
-    <row r="22" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="V21" t="s">
+        <v>350</v>
+      </c>
+      <c r="W21" t="s">
+        <v>350</v>
+      </c>
+    </row>
+    <row r="22" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A22">
         <v>16</v>
       </c>
@@ -2966,8 +3363,14 @@
       <c r="U22">
         <v>0</v>
       </c>
-    </row>
-    <row r="23" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="V22" t="s">
+        <v>361</v>
+      </c>
+      <c r="W22" t="s">
+        <v>361</v>
+      </c>
+    </row>
+    <row r="23" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A23">
         <v>16</v>
       </c>
@@ -3031,8 +3434,14 @@
       <c r="U23">
         <v>1</v>
       </c>
-    </row>
-    <row r="24" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="V23" t="s">
+        <v>347</v>
+      </c>
+      <c r="W23" t="s">
+        <v>346</v>
+      </c>
+    </row>
+    <row r="24" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A24">
         <v>16</v>
       </c>
@@ -3096,8 +3505,14 @@
       <c r="U24">
         <v>0</v>
       </c>
-    </row>
-    <row r="25" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="V24" t="s">
+        <v>346</v>
+      </c>
+      <c r="W24" t="s">
+        <v>347</v>
+      </c>
+    </row>
+    <row r="25" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A25">
         <v>16</v>
       </c>
@@ -3161,8 +3576,14 @@
       <c r="U25">
         <v>1</v>
       </c>
-    </row>
-    <row r="26" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="V25" t="s">
+        <v>357</v>
+      </c>
+      <c r="W25" t="s">
+        <v>358</v>
+      </c>
+    </row>
+    <row r="26" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A26">
         <v>16</v>
       </c>
@@ -3226,8 +3647,14 @@
       <c r="U26">
         <v>1</v>
       </c>
-    </row>
-    <row r="27" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="V26" t="s">
+        <v>346</v>
+      </c>
+      <c r="W26" t="s">
+        <v>347</v>
+      </c>
+    </row>
+    <row r="27" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A27">
         <v>16</v>
       </c>
@@ -3291,8 +3718,14 @@
       <c r="U27">
         <v>0</v>
       </c>
-    </row>
-    <row r="28" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="V27" t="s">
+        <v>346</v>
+      </c>
+      <c r="W27" t="s">
+        <v>347</v>
+      </c>
+    </row>
+    <row r="28" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A28">
         <v>16</v>
       </c>
@@ -3356,8 +3789,14 @@
       <c r="U28">
         <v>0</v>
       </c>
-    </row>
-    <row r="29" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="V28" t="s">
+        <v>346</v>
+      </c>
+      <c r="W28" t="s">
+        <v>347</v>
+      </c>
+    </row>
+    <row r="29" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A29">
         <v>16</v>
       </c>
@@ -3421,8 +3860,14 @@
       <c r="U29">
         <v>1</v>
       </c>
-    </row>
-    <row r="30" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="V29" t="s">
+        <v>346</v>
+      </c>
+      <c r="W29" t="s">
+        <v>347</v>
+      </c>
+    </row>
+    <row r="30" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A30">
         <v>16</v>
       </c>
@@ -3486,8 +3931,14 @@
       <c r="U30">
         <v>2</v>
       </c>
-    </row>
-    <row r="31" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="V30" t="s">
+        <v>346</v>
+      </c>
+      <c r="W30" t="s">
+        <v>347</v>
+      </c>
+    </row>
+    <row r="31" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A31">
         <v>16</v>
       </c>
@@ -3551,8 +4002,14 @@
       <c r="U31">
         <v>0</v>
       </c>
-    </row>
-    <row r="32" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="V31" t="s">
+        <v>357</v>
+      </c>
+      <c r="W31" t="s">
+        <v>358</v>
+      </c>
+    </row>
+    <row r="32" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A32">
         <v>17</v>
       </c>
@@ -3616,8 +4073,14 @@
       <c r="U32">
         <v>0</v>
       </c>
-    </row>
-    <row r="33" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="V32" t="s">
+        <v>362</v>
+      </c>
+      <c r="W32" t="s">
+        <v>363</v>
+      </c>
+    </row>
+    <row r="33" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A33">
         <v>17</v>
       </c>
@@ -3681,8 +4144,14 @@
       <c r="U33">
         <v>0</v>
       </c>
-    </row>
-    <row r="34" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="V33" t="s">
+        <v>351</v>
+      </c>
+      <c r="W33" t="s">
+        <v>352</v>
+      </c>
+    </row>
+    <row r="34" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A34">
         <v>17</v>
       </c>
@@ -3746,8 +4215,14 @@
       <c r="U34">
         <v>0</v>
       </c>
-    </row>
-    <row r="35" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="V34" t="s">
+        <v>346</v>
+      </c>
+      <c r="W34" t="s">
+        <v>347</v>
+      </c>
+    </row>
+    <row r="35" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A35">
         <v>17</v>
       </c>
@@ -3811,8 +4286,14 @@
       <c r="U35">
         <v>0</v>
       </c>
-    </row>
-    <row r="36" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="V35" t="s">
+        <v>364</v>
+      </c>
+      <c r="W35" t="s">
+        <v>365</v>
+      </c>
+    </row>
+    <row r="36" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A36">
         <v>17</v>
       </c>
@@ -3876,8 +4357,14 @@
       <c r="U36">
         <v>0</v>
       </c>
-    </row>
-    <row r="37" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="V36" t="s">
+        <v>346</v>
+      </c>
+      <c r="W36" t="s">
+        <v>347</v>
+      </c>
+    </row>
+    <row r="37" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A37">
         <v>17</v>
       </c>
@@ -3941,8 +4428,14 @@
       <c r="U37">
         <v>0</v>
       </c>
-    </row>
-    <row r="38" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="V37" t="s">
+        <v>346</v>
+      </c>
+      <c r="W37" t="s">
+        <v>347</v>
+      </c>
+    </row>
+    <row r="38" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A38">
         <v>17</v>
       </c>
@@ -4006,8 +4499,14 @@
       <c r="U38">
         <v>1</v>
       </c>
-    </row>
-    <row r="39" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="V38" t="s">
+        <v>350</v>
+      </c>
+      <c r="W38" t="s">
+        <v>350</v>
+      </c>
+    </row>
+    <row r="39" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A39">
         <v>18</v>
       </c>
@@ -4071,8 +4570,14 @@
       <c r="U39">
         <v>0</v>
       </c>
-    </row>
-    <row r="40" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="V39" t="s">
+        <v>366</v>
+      </c>
+      <c r="W39" t="s">
+        <v>367</v>
+      </c>
+    </row>
+    <row r="40" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A40">
         <v>18</v>
       </c>
@@ -4136,8 +4641,14 @@
       <c r="U40">
         <v>0</v>
       </c>
-    </row>
-    <row r="41" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="V40" t="s">
+        <v>346</v>
+      </c>
+      <c r="W40" t="s">
+        <v>347</v>
+      </c>
+    </row>
+    <row r="41" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A41">
         <v>18</v>
       </c>
@@ -4201,8 +4712,14 @@
       <c r="U41">
         <v>0</v>
       </c>
-    </row>
-    <row r="42" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="V41" t="s">
+        <v>346</v>
+      </c>
+      <c r="W41" t="s">
+        <v>347</v>
+      </c>
+    </row>
+    <row r="42" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A42">
         <v>18</v>
       </c>
@@ -4266,8 +4783,14 @@
       <c r="U42">
         <v>0</v>
       </c>
-    </row>
-    <row r="43" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="V42" t="s">
+        <v>368</v>
+      </c>
+      <c r="W42" t="s">
+        <v>369</v>
+      </c>
+    </row>
+    <row r="43" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A43">
         <v>18</v>
       </c>
@@ -4331,8 +4854,14 @@
       <c r="U43">
         <v>0</v>
       </c>
-    </row>
-    <row r="44" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="V43" t="s">
+        <v>370</v>
+      </c>
+      <c r="W43" t="s">
+        <v>371</v>
+      </c>
+    </row>
+    <row r="44" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A44">
         <v>18</v>
       </c>
@@ -4396,8 +4925,14 @@
       <c r="U44">
         <v>1</v>
       </c>
-    </row>
-    <row r="45" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="V44" t="s">
+        <v>355</v>
+      </c>
+      <c r="W44" t="s">
+        <v>356</v>
+      </c>
+    </row>
+    <row r="45" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A45">
         <v>18</v>
       </c>
@@ -4461,8 +4996,14 @@
       <c r="U45">
         <v>0</v>
       </c>
-    </row>
-    <row r="46" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="V45" t="s">
+        <v>351</v>
+      </c>
+      <c r="W45" t="s">
+        <v>352</v>
+      </c>
+    </row>
+    <row r="46" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A46">
         <v>18</v>
       </c>
@@ -4526,8 +5067,14 @@
       <c r="U46">
         <v>0</v>
       </c>
-    </row>
-    <row r="47" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="V46" t="s">
+        <v>350</v>
+      </c>
+      <c r="W46" t="s">
+        <v>350</v>
+      </c>
+    </row>
+    <row r="47" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A47">
         <v>19</v>
       </c>
@@ -4591,8 +5138,14 @@
       <c r="U47">
         <v>0</v>
       </c>
-    </row>
-    <row r="48" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="V47" t="s">
+        <v>372</v>
+      </c>
+      <c r="W47" t="s">
+        <v>373</v>
+      </c>
+    </row>
+    <row r="48" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A48">
         <v>19</v>
       </c>
@@ -4656,8 +5209,14 @@
       <c r="U48">
         <v>0</v>
       </c>
-    </row>
-    <row r="49" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="V48" t="s">
+        <v>346</v>
+      </c>
+      <c r="W48" t="s">
+        <v>347</v>
+      </c>
+    </row>
+    <row r="49" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A49">
         <v>19</v>
       </c>
@@ -4721,8 +5280,14 @@
       <c r="U49">
         <v>0</v>
       </c>
-    </row>
-    <row r="50" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="V49" t="s">
+        <v>346</v>
+      </c>
+      <c r="W49" t="s">
+        <v>347</v>
+      </c>
+    </row>
+    <row r="50" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A50">
         <v>19</v>
       </c>
@@ -4786,8 +5351,14 @@
       <c r="U50">
         <v>0</v>
       </c>
-    </row>
-    <row r="51" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="V50" t="s">
+        <v>346</v>
+      </c>
+      <c r="W50" t="s">
+        <v>347</v>
+      </c>
+    </row>
+    <row r="51" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A51">
         <v>19</v>
       </c>
@@ -4851,8 +5422,14 @@
       <c r="U51">
         <v>0</v>
       </c>
-    </row>
-    <row r="52" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="V51" t="s">
+        <v>346</v>
+      </c>
+      <c r="W51" t="s">
+        <v>347</v>
+      </c>
+    </row>
+    <row r="52" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A52">
         <v>19</v>
       </c>
@@ -4916,8 +5493,14 @@
       <c r="U52">
         <v>0</v>
       </c>
-    </row>
-    <row r="53" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="V52" t="s">
+        <v>359</v>
+      </c>
+      <c r="W52" t="s">
+        <v>360</v>
+      </c>
+    </row>
+    <row r="53" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A53">
         <v>1</v>
       </c>
@@ -4981,8 +5564,14 @@
       <c r="U53">
         <v>0</v>
       </c>
-    </row>
-    <row r="54" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="V53" t="s">
+        <v>350</v>
+      </c>
+      <c r="W53" t="s">
+        <v>350</v>
+      </c>
+    </row>
+    <row r="54" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A54">
         <v>21</v>
       </c>
@@ -5046,8 +5635,14 @@
       <c r="U54">
         <v>0</v>
       </c>
-    </row>
-    <row r="55" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="V54" t="s">
+        <v>346</v>
+      </c>
+      <c r="W54" t="s">
+        <v>347</v>
+      </c>
+    </row>
+    <row r="55" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A55">
         <v>21</v>
       </c>
@@ -5111,8 +5706,14 @@
       <c r="U55">
         <v>0</v>
       </c>
-    </row>
-    <row r="56" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="V55" t="s">
+        <v>357</v>
+      </c>
+      <c r="W55" t="s">
+        <v>358</v>
+      </c>
+    </row>
+    <row r="56" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A56">
         <v>21</v>
       </c>
@@ -5176,8 +5777,14 @@
       <c r="U56">
         <v>0</v>
       </c>
-    </row>
-    <row r="57" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="V56" t="s">
+        <v>374</v>
+      </c>
+      <c r="W56" t="s">
+        <v>375</v>
+      </c>
+    </row>
+    <row r="57" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A57">
         <v>21</v>
       </c>
@@ -5241,8 +5848,14 @@
       <c r="U57">
         <v>0</v>
       </c>
-    </row>
-    <row r="58" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="V57" t="s">
+        <v>346</v>
+      </c>
+      <c r="W57" t="s">
+        <v>347</v>
+      </c>
+    </row>
+    <row r="58" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A58">
         <v>21</v>
       </c>
@@ -5306,8 +5919,14 @@
       <c r="U58">
         <v>1</v>
       </c>
-    </row>
-    <row r="59" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="V58" t="s">
+        <v>376</v>
+      </c>
+      <c r="W58" t="s">
+        <v>377</v>
+      </c>
+    </row>
+    <row r="59" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A59">
         <v>21</v>
       </c>
@@ -5371,8 +5990,14 @@
       <c r="U59">
         <v>0</v>
       </c>
-    </row>
-    <row r="60" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="V59" t="s">
+        <v>378</v>
+      </c>
+      <c r="W59" t="s">
+        <v>379</v>
+      </c>
+    </row>
+    <row r="60" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A60">
         <v>21</v>
       </c>
@@ -5436,8 +6061,14 @@
       <c r="U60">
         <v>0</v>
       </c>
-    </row>
-    <row r="61" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="V60" t="s">
+        <v>350</v>
+      </c>
+      <c r="W60" t="s">
+        <v>350</v>
+      </c>
+    </row>
+    <row r="61" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A61">
         <v>22</v>
       </c>
@@ -5501,8 +6132,14 @@
       <c r="U61">
         <v>0</v>
       </c>
-    </row>
-    <row r="62" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="V61" t="s">
+        <v>350</v>
+      </c>
+      <c r="W61" t="s">
+        <v>350</v>
+      </c>
+    </row>
+    <row r="62" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A62">
         <v>22</v>
       </c>
@@ -5566,8 +6203,14 @@
       <c r="U62">
         <v>0</v>
       </c>
-    </row>
-    <row r="63" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="V62" t="s">
+        <v>346</v>
+      </c>
+      <c r="W62" t="s">
+        <v>347</v>
+      </c>
+    </row>
+    <row r="63" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A63">
         <v>22</v>
       </c>
@@ -5631,8 +6274,14 @@
       <c r="U63">
         <v>0</v>
       </c>
-    </row>
-    <row r="64" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="V63" t="s">
+        <v>364</v>
+      </c>
+      <c r="W63" t="s">
+        <v>365</v>
+      </c>
+    </row>
+    <row r="64" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A64">
         <v>22</v>
       </c>
@@ -5696,8 +6345,14 @@
       <c r="U64">
         <v>0</v>
       </c>
-    </row>
-    <row r="65" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="V64" t="s">
+        <v>380</v>
+      </c>
+      <c r="W64" t="s">
+        <v>381</v>
+      </c>
+    </row>
+    <row r="65" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A65">
         <v>22</v>
       </c>
@@ -5761,8 +6416,14 @@
       <c r="U65">
         <v>0</v>
       </c>
-    </row>
-    <row r="66" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="V65" t="s">
+        <v>382</v>
+      </c>
+      <c r="W65" t="s">
+        <v>383</v>
+      </c>
+    </row>
+    <row r="66" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A66">
         <v>23</v>
       </c>
@@ -5826,8 +6487,14 @@
       <c r="U66">
         <v>0</v>
       </c>
-    </row>
-    <row r="67" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="V66" t="s">
+        <v>344</v>
+      </c>
+      <c r="W66" t="s">
+        <v>345</v>
+      </c>
+    </row>
+    <row r="67" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A67">
         <v>23</v>
       </c>
@@ -5891,8 +6558,14 @@
       <c r="U67">
         <v>0</v>
       </c>
-    </row>
-    <row r="68" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="V67" t="s">
+        <v>350</v>
+      </c>
+      <c r="W67" t="s">
+        <v>350</v>
+      </c>
+    </row>
+    <row r="68" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A68">
         <v>24</v>
       </c>
@@ -5956,8 +6629,14 @@
       <c r="U68">
         <v>1</v>
       </c>
-    </row>
-    <row r="69" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="V68" t="s">
+        <v>350</v>
+      </c>
+      <c r="W68" t="s">
+        <v>350</v>
+      </c>
+    </row>
+    <row r="69" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A69">
         <v>24</v>
       </c>
@@ -6021,8 +6700,14 @@
       <c r="U69">
         <v>3</v>
       </c>
-    </row>
-    <row r="70" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="V69" t="s">
+        <v>361</v>
+      </c>
+      <c r="W69" t="s">
+        <v>361</v>
+      </c>
+    </row>
+    <row r="70" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A70">
         <v>24</v>
       </c>
@@ -6086,8 +6771,14 @@
       <c r="U70">
         <v>0</v>
       </c>
-    </row>
-    <row r="71" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="V70" t="s">
+        <v>384</v>
+      </c>
+      <c r="W70" t="s">
+        <v>385</v>
+      </c>
+    </row>
+    <row r="71" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A71">
         <v>24</v>
       </c>
@@ -6151,8 +6842,14 @@
       <c r="U71">
         <v>0</v>
       </c>
-    </row>
-    <row r="72" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="V71" t="s">
+        <v>357</v>
+      </c>
+      <c r="W71" t="s">
+        <v>358</v>
+      </c>
+    </row>
+    <row r="72" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A72">
         <v>24</v>
       </c>
@@ -6216,8 +6913,14 @@
       <c r="U72">
         <v>0</v>
       </c>
-    </row>
-    <row r="73" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="V72" t="s">
+        <v>355</v>
+      </c>
+      <c r="W72" t="s">
+        <v>356</v>
+      </c>
+    </row>
+    <row r="73" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A73">
         <v>25</v>
       </c>
@@ -6281,8 +6984,14 @@
       <c r="U73">
         <v>0</v>
       </c>
-    </row>
-    <row r="74" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="V73" t="s">
+        <v>386</v>
+      </c>
+      <c r="W73" t="s">
+        <v>387</v>
+      </c>
+    </row>
+    <row r="74" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A74">
         <v>25</v>
       </c>
@@ -6346,8 +7055,14 @@
       <c r="U74">
         <v>1</v>
       </c>
-    </row>
-    <row r="75" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="V74" t="s">
+        <v>346</v>
+      </c>
+      <c r="W74" t="s">
+        <v>347</v>
+      </c>
+    </row>
+    <row r="75" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A75">
         <v>25</v>
       </c>
@@ -6411,8 +7126,14 @@
       <c r="U75">
         <v>0</v>
       </c>
-    </row>
-    <row r="76" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="V75" t="s">
+        <v>346</v>
+      </c>
+      <c r="W75" t="s">
+        <v>347</v>
+      </c>
+    </row>
+    <row r="76" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A76">
         <v>25</v>
       </c>
@@ -6476,8 +7197,14 @@
       <c r="U76">
         <v>0</v>
       </c>
-    </row>
-    <row r="77" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="V76" t="s">
+        <v>346</v>
+      </c>
+      <c r="W76" t="s">
+        <v>347</v>
+      </c>
+    </row>
+    <row r="77" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A77">
         <v>25</v>
       </c>
@@ -6541,8 +7268,14 @@
       <c r="U77">
         <v>0</v>
       </c>
-    </row>
-    <row r="78" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="V77" t="s">
+        <v>362</v>
+      </c>
+      <c r="W77" t="s">
+        <v>363</v>
+      </c>
+    </row>
+    <row r="78" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A78">
         <v>25</v>
       </c>
@@ -6606,8 +7339,14 @@
       <c r="U78">
         <v>0</v>
       </c>
-    </row>
-    <row r="79" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="V78" t="s">
+        <v>388</v>
+      </c>
+      <c r="W78" t="s">
+        <v>389</v>
+      </c>
+    </row>
+    <row r="79" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A79">
         <v>26</v>
       </c>
@@ -6671,8 +7410,14 @@
       <c r="U79">
         <v>1</v>
       </c>
-    </row>
-    <row r="80" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="V79" t="s">
+        <v>346</v>
+      </c>
+      <c r="W79" t="s">
+        <v>347</v>
+      </c>
+    </row>
+    <row r="80" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A80">
         <v>26</v>
       </c>
@@ -6736,8 +7481,14 @@
       <c r="U80">
         <v>1</v>
       </c>
-    </row>
-    <row r="81" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="V80" t="s">
+        <v>350</v>
+      </c>
+      <c r="W80" t="s">
+        <v>350</v>
+      </c>
+    </row>
+    <row r="81" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A81">
         <v>26</v>
       </c>
@@ -6801,8 +7552,14 @@
       <c r="U81">
         <v>0</v>
       </c>
-    </row>
-    <row r="82" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="V81" t="s">
+        <v>359</v>
+      </c>
+      <c r="W81" t="s">
+        <v>360</v>
+      </c>
+    </row>
+    <row r="82" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A82">
         <v>26</v>
       </c>
@@ -6866,8 +7623,14 @@
       <c r="U82">
         <v>2</v>
       </c>
-    </row>
-    <row r="83" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="V82" t="s">
+        <v>390</v>
+      </c>
+      <c r="W82" t="s">
+        <v>391</v>
+      </c>
+    </row>
+    <row r="83" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A83">
         <v>26</v>
       </c>
@@ -6931,8 +7694,14 @@
       <c r="U83">
         <v>0</v>
       </c>
-    </row>
-    <row r="84" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="V83" t="s">
+        <v>350</v>
+      </c>
+      <c r="W83" t="s">
+        <v>350</v>
+      </c>
+    </row>
+    <row r="84" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A84">
         <v>27</v>
       </c>
@@ -6996,8 +7765,14 @@
       <c r="U84">
         <v>0</v>
       </c>
-    </row>
-    <row r="85" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="V84" t="s">
+        <v>368</v>
+      </c>
+      <c r="W84" t="s">
+        <v>369</v>
+      </c>
+    </row>
+    <row r="85" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A85">
         <v>27</v>
       </c>
@@ -7061,8 +7836,14 @@
       <c r="U85">
         <v>0</v>
       </c>
-    </row>
-    <row r="86" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="V85" t="s">
+        <v>350</v>
+      </c>
+      <c r="W85" t="s">
+        <v>350</v>
+      </c>
+    </row>
+    <row r="86" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A86">
         <v>27</v>
       </c>
@@ -7126,8 +7907,14 @@
       <c r="U86">
         <v>0</v>
       </c>
-    </row>
-    <row r="87" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="V86" t="s">
+        <v>346</v>
+      </c>
+      <c r="W86" t="s">
+        <v>347</v>
+      </c>
+    </row>
+    <row r="87" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A87">
         <v>27</v>
       </c>
@@ -7191,8 +7978,14 @@
       <c r="U87">
         <v>2</v>
       </c>
-    </row>
-    <row r="88" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="V87" t="s">
+        <v>346</v>
+      </c>
+      <c r="W87" t="s">
+        <v>347</v>
+      </c>
+    </row>
+    <row r="88" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A88">
         <v>27</v>
       </c>
@@ -7256,8 +8049,14 @@
       <c r="U88">
         <v>0</v>
       </c>
-    </row>
-    <row r="89" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="V88" t="s">
+        <v>392</v>
+      </c>
+      <c r="W88" t="s">
+        <v>393</v>
+      </c>
+    </row>
+    <row r="89" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A89">
         <v>27</v>
       </c>
@@ -7321,8 +8120,14 @@
       <c r="U89">
         <v>1</v>
       </c>
-    </row>
-    <row r="90" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="V89" t="s">
+        <v>350</v>
+      </c>
+      <c r="W89" t="s">
+        <v>350</v>
+      </c>
+    </row>
+    <row r="90" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A90">
         <v>27</v>
       </c>
@@ -7386,8 +8191,14 @@
       <c r="U90">
         <v>0</v>
       </c>
-    </row>
-    <row r="91" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="V90" t="s">
+        <v>394</v>
+      </c>
+      <c r="W90" t="s">
+        <v>395</v>
+      </c>
+    </row>
+    <row r="91" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A91">
         <v>2</v>
       </c>
@@ -7451,8 +8262,14 @@
       <c r="U91">
         <v>0</v>
       </c>
-    </row>
-    <row r="92" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="V91" t="s">
+        <v>396</v>
+      </c>
+      <c r="W91" t="s">
+        <v>397</v>
+      </c>
+    </row>
+    <row r="92" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A92">
         <v>2</v>
       </c>
@@ -7516,8 +8333,14 @@
       <c r="U92">
         <v>1</v>
       </c>
-    </row>
-    <row r="93" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="V92" t="s">
+        <v>346</v>
+      </c>
+      <c r="W92" t="s">
+        <v>347</v>
+      </c>
+    </row>
+    <row r="93" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A93">
         <v>30</v>
       </c>
@@ -7581,8 +8404,14 @@
       <c r="U93">
         <v>0</v>
       </c>
-    </row>
-    <row r="94" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="V93" t="s">
+        <v>346</v>
+      </c>
+      <c r="W93" t="s">
+        <v>347</v>
+      </c>
+    </row>
+    <row r="94" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A94">
         <v>30</v>
       </c>
@@ -7646,8 +8475,14 @@
       <c r="U94">
         <v>0</v>
       </c>
-    </row>
-    <row r="95" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="V94" t="s">
+        <v>346</v>
+      </c>
+      <c r="W94" t="s">
+        <v>347</v>
+      </c>
+    </row>
+    <row r="95" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A95">
         <v>30</v>
       </c>
@@ -7711,8 +8546,14 @@
       <c r="U95">
         <v>0</v>
       </c>
-    </row>
-    <row r="96" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="V95" t="s">
+        <v>390</v>
+      </c>
+      <c r="W95" t="s">
+        <v>391</v>
+      </c>
+    </row>
+    <row r="96" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A96">
         <v>30</v>
       </c>
@@ -7776,8 +8617,14 @@
       <c r="U96">
         <v>0</v>
       </c>
-    </row>
-    <row r="97" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="V96" t="s">
+        <v>351</v>
+      </c>
+      <c r="W96" t="s">
+        <v>352</v>
+      </c>
+    </row>
+    <row r="97" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A97">
         <v>30</v>
       </c>
@@ -7841,8 +8688,14 @@
       <c r="U97">
         <v>0</v>
       </c>
-    </row>
-    <row r="98" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="V97" t="s">
+        <v>346</v>
+      </c>
+      <c r="W97" t="s">
+        <v>347</v>
+      </c>
+    </row>
+    <row r="98" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A98">
         <v>30</v>
       </c>
@@ -7906,8 +8759,14 @@
       <c r="U98">
         <v>2</v>
       </c>
-    </row>
-    <row r="99" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="V98" t="s">
+        <v>398</v>
+      </c>
+      <c r="W98" t="s">
+        <v>399</v>
+      </c>
+    </row>
+    <row r="99" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A99">
         <v>30</v>
       </c>
@@ -7971,8 +8830,14 @@
       <c r="U99">
         <v>0</v>
       </c>
-    </row>
-    <row r="100" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="V99" t="s">
+        <v>350</v>
+      </c>
+      <c r="W99" t="s">
+        <v>350</v>
+      </c>
+    </row>
+    <row r="100" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A100">
         <v>30</v>
       </c>
@@ -8036,8 +8901,14 @@
       <c r="U100">
         <v>0</v>
       </c>
-    </row>
-    <row r="101" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="V100" t="s">
+        <v>351</v>
+      </c>
+      <c r="W100" t="s">
+        <v>352</v>
+      </c>
+    </row>
+    <row r="101" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A101">
         <v>31</v>
       </c>
@@ -8101,8 +8972,14 @@
       <c r="U101">
         <v>0</v>
       </c>
-    </row>
-    <row r="102" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="V101" t="s">
+        <v>346</v>
+      </c>
+      <c r="W101" t="s">
+        <v>347</v>
+      </c>
+    </row>
+    <row r="102" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A102">
         <v>31</v>
       </c>
@@ -8166,8 +9043,14 @@
       <c r="U102">
         <v>3</v>
       </c>
-    </row>
-    <row r="103" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="V102" t="s">
+        <v>364</v>
+      </c>
+      <c r="W102" t="s">
+        <v>365</v>
+      </c>
+    </row>
+    <row r="103" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A103">
         <v>31</v>
       </c>
@@ -8231,8 +9114,14 @@
       <c r="U103">
         <v>0</v>
       </c>
-    </row>
-    <row r="104" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="V103" t="s">
+        <v>346</v>
+      </c>
+      <c r="W103" t="s">
+        <v>347</v>
+      </c>
+    </row>
+    <row r="104" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A104">
         <v>31</v>
       </c>
@@ -8296,8 +9185,14 @@
       <c r="U104">
         <v>3</v>
       </c>
-    </row>
-    <row r="105" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="V104" t="s">
+        <v>400</v>
+      </c>
+      <c r="W104" t="s">
+        <v>401</v>
+      </c>
+    </row>
+    <row r="105" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A105">
         <v>32</v>
       </c>
@@ -8361,8 +9256,14 @@
       <c r="U105">
         <v>0</v>
       </c>
-    </row>
-    <row r="106" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="V105" t="s">
+        <v>402</v>
+      </c>
+      <c r="W105" t="s">
+        <v>403</v>
+      </c>
+    </row>
+    <row r="106" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A106">
         <v>32</v>
       </c>
@@ -8426,8 +9327,14 @@
       <c r="U106">
         <v>1</v>
       </c>
-    </row>
-    <row r="107" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="V106" t="s">
+        <v>376</v>
+      </c>
+      <c r="W106" t="s">
+        <v>377</v>
+      </c>
+    </row>
+    <row r="107" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A107">
         <v>32</v>
       </c>
@@ -8491,8 +9398,14 @@
       <c r="U107">
         <v>0</v>
       </c>
-    </row>
-    <row r="108" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="V107" t="s">
+        <v>346</v>
+      </c>
+      <c r="W107" t="s">
+        <v>347</v>
+      </c>
+    </row>
+    <row r="108" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A108">
         <v>32</v>
       </c>
@@ -8556,8 +9469,14 @@
       <c r="U108">
         <v>0</v>
       </c>
-    </row>
-    <row r="109" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="V108" t="s">
+        <v>357</v>
+      </c>
+      <c r="W108" t="s">
+        <v>358</v>
+      </c>
+    </row>
+    <row r="109" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A109">
         <v>32</v>
       </c>
@@ -8621,8 +9540,14 @@
       <c r="U109">
         <v>0</v>
       </c>
-    </row>
-    <row r="110" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="V109" t="s">
+        <v>346</v>
+      </c>
+      <c r="W109" t="s">
+        <v>347</v>
+      </c>
+    </row>
+    <row r="110" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A110">
         <v>33</v>
       </c>
@@ -8686,8 +9611,14 @@
       <c r="U110">
         <v>0</v>
       </c>
-    </row>
-    <row r="111" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="V110" t="s">
+        <v>350</v>
+      </c>
+      <c r="W110" t="s">
+        <v>350</v>
+      </c>
+    </row>
+    <row r="111" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A111">
         <v>34</v>
       </c>
@@ -8751,8 +9682,14 @@
       <c r="U111">
         <v>0</v>
       </c>
-    </row>
-    <row r="112" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="V111" t="s">
+        <v>350</v>
+      </c>
+      <c r="W111" t="s">
+        <v>350</v>
+      </c>
+    </row>
+    <row r="112" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A112">
         <v>34</v>
       </c>
@@ -8816,8 +9753,14 @@
       <c r="U112">
         <v>0</v>
       </c>
-    </row>
-    <row r="113" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="V112" t="s">
+        <v>350</v>
+      </c>
+      <c r="W112" t="s">
+        <v>350</v>
+      </c>
+    </row>
+    <row r="113" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A113">
         <v>34</v>
       </c>
@@ -8881,8 +9824,14 @@
       <c r="U113">
         <v>0</v>
       </c>
-    </row>
-    <row r="114" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="V113" t="s">
+        <v>350</v>
+      </c>
+      <c r="W113" t="s">
+        <v>350</v>
+      </c>
+    </row>
+    <row r="114" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A114">
         <v>35</v>
       </c>
@@ -8946,8 +9895,14 @@
       <c r="U114">
         <v>0</v>
       </c>
-    </row>
-    <row r="115" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="V114" t="s">
+        <v>350</v>
+      </c>
+      <c r="W114" t="s">
+        <v>350</v>
+      </c>
+    </row>
+    <row r="115" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A115">
         <v>35</v>
       </c>
@@ -9011,8 +9966,14 @@
       <c r="U115">
         <v>0</v>
       </c>
-    </row>
-    <row r="116" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="V115" t="s">
+        <v>350</v>
+      </c>
+      <c r="W115" t="s">
+        <v>350</v>
+      </c>
+    </row>
+    <row r="116" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A116">
         <v>35</v>
       </c>
@@ -9076,8 +10037,14 @@
       <c r="U116">
         <v>0</v>
       </c>
-    </row>
-    <row r="117" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="V116" t="s">
+        <v>350</v>
+      </c>
+      <c r="W116" t="s">
+        <v>350</v>
+      </c>
+    </row>
+    <row r="117" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A117">
         <v>35</v>
       </c>
@@ -9141,8 +10108,14 @@
       <c r="U117">
         <v>4</v>
       </c>
-    </row>
-    <row r="118" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="V117" t="s">
+        <v>350</v>
+      </c>
+      <c r="W117" t="s">
+        <v>350</v>
+      </c>
+    </row>
+    <row r="118" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A118">
         <v>35</v>
       </c>
@@ -9206,8 +10179,14 @@
       <c r="U118">
         <v>0</v>
       </c>
-    </row>
-    <row r="119" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="V118" t="s">
+        <v>351</v>
+      </c>
+      <c r="W118" t="s">
+        <v>352</v>
+      </c>
+    </row>
+    <row r="119" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A119">
         <v>35</v>
       </c>
@@ -9271,8 +10250,14 @@
       <c r="U119">
         <v>1</v>
       </c>
-    </row>
-    <row r="120" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="V119" t="s">
+        <v>364</v>
+      </c>
+      <c r="W119" t="s">
+        <v>365</v>
+      </c>
+    </row>
+    <row r="120" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A120">
         <v>35</v>
       </c>
@@ -9336,8 +10321,14 @@
       <c r="U120">
         <v>0</v>
       </c>
-    </row>
-    <row r="121" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="V120" t="s">
+        <v>390</v>
+      </c>
+      <c r="W120" t="s">
+        <v>391</v>
+      </c>
+    </row>
+    <row r="121" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A121">
         <v>35</v>
       </c>
@@ -9401,8 +10392,14 @@
       <c r="U121">
         <v>1</v>
       </c>
-    </row>
-    <row r="122" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="V121" t="s">
+        <v>357</v>
+      </c>
+      <c r="W121" t="s">
+        <v>358</v>
+      </c>
+    </row>
+    <row r="122" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A122">
         <v>35</v>
       </c>
@@ -9466,8 +10463,14 @@
       <c r="U122">
         <v>0</v>
       </c>
-    </row>
-    <row r="123" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="V122" t="s">
+        <v>346</v>
+      </c>
+      <c r="W122" t="s">
+        <v>347</v>
+      </c>
+    </row>
+    <row r="123" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A123">
         <v>35</v>
       </c>
@@ -9531,8 +10534,14 @@
       <c r="U123">
         <v>0</v>
       </c>
-    </row>
-    <row r="124" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="V123" t="s">
+        <v>346</v>
+      </c>
+      <c r="W123" t="s">
+        <v>347</v>
+      </c>
+    </row>
+    <row r="124" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A124">
         <v>37</v>
       </c>
@@ -9596,8 +10605,14 @@
       <c r="U124">
         <v>0</v>
       </c>
-    </row>
-    <row r="125" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="V124" t="s">
+        <v>346</v>
+      </c>
+      <c r="W124" t="s">
+        <v>347</v>
+      </c>
+    </row>
+    <row r="125" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A125">
         <v>37</v>
       </c>
@@ -9661,8 +10676,14 @@
       <c r="U125">
         <v>0</v>
       </c>
-    </row>
-    <row r="126" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="V125" t="s">
+        <v>392</v>
+      </c>
+      <c r="W125" t="s">
+        <v>393</v>
+      </c>
+    </row>
+    <row r="126" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A126">
         <v>37</v>
       </c>
@@ -9726,8 +10747,14 @@
       <c r="U126">
         <v>0</v>
       </c>
-    </row>
-    <row r="127" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="V126" t="s">
+        <v>346</v>
+      </c>
+      <c r="W126" t="s">
+        <v>347</v>
+      </c>
+    </row>
+    <row r="127" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A127">
         <v>37</v>
       </c>
@@ -9791,8 +10818,14 @@
       <c r="U127">
         <v>1</v>
       </c>
-    </row>
-    <row r="128" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="V127" t="s">
+        <v>392</v>
+      </c>
+      <c r="W127" t="s">
+        <v>393</v>
+      </c>
+    </row>
+    <row r="128" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A128">
         <v>37</v>
       </c>
@@ -9856,8 +10889,14 @@
       <c r="U128">
         <v>0</v>
       </c>
-    </row>
-    <row r="129" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="V128" t="s">
+        <v>368</v>
+      </c>
+      <c r="W128" t="s">
+        <v>369</v>
+      </c>
+    </row>
+    <row r="129" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A129">
         <v>37</v>
       </c>
@@ -9921,8 +10960,14 @@
       <c r="U129">
         <v>0</v>
       </c>
-    </row>
-    <row r="130" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="V129" t="s">
+        <v>346</v>
+      </c>
+      <c r="W129" t="s">
+        <v>347</v>
+      </c>
+    </row>
+    <row r="130" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A130">
         <v>37</v>
       </c>
@@ -9986,8 +11031,14 @@
       <c r="U130">
         <v>0</v>
       </c>
-    </row>
-    <row r="131" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="V130" t="s">
+        <v>370</v>
+      </c>
+      <c r="W130" t="s">
+        <v>371</v>
+      </c>
+    </row>
+    <row r="131" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A131">
         <v>37</v>
       </c>
@@ -10051,8 +11102,14 @@
       <c r="U131">
         <v>2</v>
       </c>
-    </row>
-    <row r="132" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="V131" t="s">
+        <v>346</v>
+      </c>
+      <c r="W131" t="s">
+        <v>347</v>
+      </c>
+    </row>
+    <row r="132" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A132">
         <v>37</v>
       </c>
@@ -10116,8 +11173,14 @@
       <c r="U132">
         <v>0</v>
       </c>
-    </row>
-    <row r="133" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="V132" t="s">
+        <v>346</v>
+      </c>
+      <c r="W132" t="s">
+        <v>347</v>
+      </c>
+    </row>
+    <row r="133" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A133">
         <v>37</v>
       </c>
@@ -10181,8 +11244,14 @@
       <c r="U133">
         <v>0</v>
       </c>
-    </row>
-    <row r="134" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="V133" t="s">
+        <v>346</v>
+      </c>
+      <c r="W133" t="s">
+        <v>347</v>
+      </c>
+    </row>
+    <row r="134" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A134">
         <v>37</v>
       </c>
@@ -10246,8 +11315,14 @@
       <c r="U134">
         <v>0</v>
       </c>
-    </row>
-    <row r="135" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="V134" t="s">
+        <v>346</v>
+      </c>
+      <c r="W134" t="s">
+        <v>347</v>
+      </c>
+    </row>
+    <row r="135" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A135">
         <v>3</v>
       </c>
@@ -10311,8 +11386,14 @@
       <c r="U135">
         <v>0</v>
       </c>
-    </row>
-    <row r="136" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="V135" t="s">
+        <v>350</v>
+      </c>
+      <c r="W135" t="s">
+        <v>350</v>
+      </c>
+    </row>
+    <row r="136" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A136">
         <v>3</v>
       </c>
@@ -10376,8 +11457,14 @@
       <c r="U136">
         <v>0</v>
       </c>
-    </row>
-    <row r="137" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="V136" t="s">
+        <v>350</v>
+      </c>
+      <c r="W136" t="s">
+        <v>350</v>
+      </c>
+    </row>
+    <row r="137" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A137">
         <v>41</v>
       </c>
@@ -10441,8 +11528,14 @@
       <c r="U137">
         <v>0</v>
       </c>
-    </row>
-    <row r="138" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="V137" t="s">
+        <v>357</v>
+      </c>
+      <c r="W137" t="s">
+        <v>358</v>
+      </c>
+    </row>
+    <row r="138" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A138">
         <v>41</v>
       </c>
@@ -10506,8 +11599,14 @@
       <c r="U138">
         <v>1</v>
       </c>
-    </row>
-    <row r="139" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="V138" t="s">
+        <v>346</v>
+      </c>
+      <c r="W138" t="s">
+        <v>347</v>
+      </c>
+    </row>
+    <row r="139" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A139">
         <v>41</v>
       </c>
@@ -10571,8 +11670,14 @@
       <c r="U139">
         <v>0</v>
       </c>
-    </row>
-    <row r="140" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="V139" t="s">
+        <v>344</v>
+      </c>
+      <c r="W139" t="s">
+        <v>345</v>
+      </c>
+    </row>
+    <row r="140" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A140">
         <v>41</v>
       </c>
@@ -10636,8 +11741,14 @@
       <c r="U140">
         <v>0</v>
       </c>
-    </row>
-    <row r="141" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="V140" t="s">
+        <v>350</v>
+      </c>
+      <c r="W140" t="s">
+        <v>350</v>
+      </c>
+    </row>
+    <row r="141" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A141">
         <v>42</v>
       </c>
@@ -10701,8 +11812,14 @@
       <c r="U141">
         <v>0</v>
       </c>
-    </row>
-    <row r="142" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="V141" t="s">
+        <v>350</v>
+      </c>
+      <c r="W141" t="s">
+        <v>350</v>
+      </c>
+    </row>
+    <row r="142" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A142">
         <v>42</v>
       </c>
@@ -10766,8 +11883,14 @@
       <c r="U142">
         <v>2</v>
       </c>
-    </row>
-    <row r="143" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="V142" t="s">
+        <v>350</v>
+      </c>
+      <c r="W142" t="s">
+        <v>350</v>
+      </c>
+    </row>
+    <row r="143" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A143">
         <v>42</v>
       </c>
@@ -10831,8 +11954,14 @@
       <c r="U143">
         <v>0</v>
       </c>
-    </row>
-    <row r="144" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="V143" t="s">
+        <v>350</v>
+      </c>
+      <c r="W143" t="s">
+        <v>350</v>
+      </c>
+    </row>
+    <row r="144" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A144">
         <v>43</v>
       </c>
@@ -10896,8 +12025,14 @@
       <c r="U144">
         <v>0</v>
       </c>
-    </row>
-    <row r="145" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="V144" t="s">
+        <v>364</v>
+      </c>
+      <c r="W144" t="s">
+        <v>365</v>
+      </c>
+    </row>
+    <row r="145" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A145">
         <v>43</v>
       </c>
@@ -10961,8 +12096,14 @@
       <c r="U145">
         <v>0</v>
       </c>
-    </row>
-    <row r="146" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="V145" t="s">
+        <v>372</v>
+      </c>
+      <c r="W145" t="s">
+        <v>373</v>
+      </c>
+    </row>
+    <row r="146" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A146">
         <v>43</v>
       </c>
@@ -11026,8 +12167,14 @@
       <c r="U146">
         <v>2</v>
       </c>
-    </row>
-    <row r="147" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="V146" t="s">
+        <v>355</v>
+      </c>
+      <c r="W146" t="s">
+        <v>356</v>
+      </c>
+    </row>
+    <row r="147" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A147">
         <v>43</v>
       </c>
@@ -11091,8 +12238,14 @@
       <c r="U147">
         <v>0</v>
       </c>
-    </row>
-    <row r="148" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="V147" t="s">
+        <v>344</v>
+      </c>
+      <c r="W147" t="s">
+        <v>345</v>
+      </c>
+    </row>
+    <row r="148" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A148">
         <v>44</v>
       </c>
@@ -11156,8 +12309,14 @@
       <c r="U148">
         <v>0</v>
       </c>
-    </row>
-    <row r="149" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="V148" t="s">
+        <v>350</v>
+      </c>
+      <c r="W148" t="s">
+        <v>350</v>
+      </c>
+    </row>
+    <row r="149" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A149">
         <v>44</v>
       </c>
@@ -11221,8 +12380,14 @@
       <c r="U149">
         <v>1</v>
       </c>
-    </row>
-    <row r="150" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="V149" t="s">
+        <v>350</v>
+      </c>
+      <c r="W149" t="s">
+        <v>350</v>
+      </c>
+    </row>
+    <row r="150" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A150">
         <v>45</v>
       </c>
@@ -11286,8 +12451,14 @@
       <c r="U150">
         <v>1</v>
       </c>
-    </row>
-    <row r="151" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="V150" t="s">
+        <v>346</v>
+      </c>
+      <c r="W150" t="s">
+        <v>347</v>
+      </c>
+    </row>
+    <row r="151" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A151">
         <v>45</v>
       </c>
@@ -11351,8 +12522,14 @@
       <c r="U151">
         <v>4</v>
       </c>
-    </row>
-    <row r="152" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="V151" t="s">
+        <v>347</v>
+      </c>
+      <c r="W151" t="s">
+        <v>346</v>
+      </c>
+    </row>
+    <row r="152" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A152">
         <v>45</v>
       </c>
@@ -11416,8 +12593,14 @@
       <c r="U152">
         <v>0</v>
       </c>
-    </row>
-    <row r="153" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="V152" t="s">
+        <v>359</v>
+      </c>
+      <c r="W152" t="s">
+        <v>360</v>
+      </c>
+    </row>
+    <row r="153" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A153">
         <v>45</v>
       </c>
@@ -11481,8 +12664,14 @@
       <c r="U153">
         <v>6</v>
       </c>
-    </row>
-    <row r="154" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="V153" t="s">
+        <v>404</v>
+      </c>
+      <c r="W153" t="s">
+        <v>405</v>
+      </c>
+    </row>
+    <row r="154" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A154">
         <v>45</v>
       </c>
@@ -11546,8 +12735,14 @@
       <c r="U154">
         <v>0</v>
       </c>
-    </row>
-    <row r="155" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="V154" t="s">
+        <v>370</v>
+      </c>
+      <c r="W154" t="s">
+        <v>371</v>
+      </c>
+    </row>
+    <row r="155" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A155">
         <v>46</v>
       </c>
@@ -11611,8 +12806,14 @@
       <c r="U155">
         <v>0</v>
       </c>
-    </row>
-    <row r="156" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="V155" t="s">
+        <v>350</v>
+      </c>
+      <c r="W155" t="s">
+        <v>350</v>
+      </c>
+    </row>
+    <row r="156" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A156">
         <v>46</v>
       </c>
@@ -11676,8 +12877,14 @@
       <c r="U156">
         <v>0</v>
       </c>
-    </row>
-    <row r="157" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="V156" t="s">
+        <v>350</v>
+      </c>
+      <c r="W156" t="s">
+        <v>350</v>
+      </c>
+    </row>
+    <row r="157" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A157">
         <v>46</v>
       </c>
@@ -11741,8 +12948,14 @@
       <c r="U157">
         <v>2</v>
       </c>
-    </row>
-    <row r="158" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="V157" t="s">
+        <v>357</v>
+      </c>
+      <c r="W157" t="s">
+        <v>358</v>
+      </c>
+    </row>
+    <row r="158" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A158">
         <v>47</v>
       </c>
@@ -11806,8 +13019,14 @@
       <c r="U158">
         <v>0</v>
       </c>
-    </row>
-    <row r="159" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="V158" t="s">
+        <v>346</v>
+      </c>
+      <c r="W158" t="s">
+        <v>347</v>
+      </c>
+    </row>
+    <row r="159" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A159">
         <v>47</v>
       </c>
@@ -11871,8 +13090,14 @@
       <c r="U159">
         <v>0</v>
       </c>
-    </row>
-    <row r="160" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="V159" t="s">
+        <v>406</v>
+      </c>
+      <c r="W159" t="s">
+        <v>407</v>
+      </c>
+    </row>
+    <row r="160" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A160">
         <v>47</v>
       </c>
@@ -11936,8 +13161,14 @@
       <c r="U160">
         <v>7</v>
       </c>
-    </row>
-    <row r="161" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="V160" t="s">
+        <v>408</v>
+      </c>
+      <c r="W160" t="s">
+        <v>409</v>
+      </c>
+    </row>
+    <row r="161" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A161">
         <v>47</v>
       </c>
@@ -12001,8 +13232,14 @@
       <c r="U161">
         <v>0</v>
       </c>
-    </row>
-    <row r="162" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="V161" t="s">
+        <v>350</v>
+      </c>
+      <c r="W161" t="s">
+        <v>350</v>
+      </c>
+    </row>
+    <row r="162" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A162">
         <v>48</v>
       </c>
@@ -12066,8 +13303,14 @@
       <c r="U162">
         <v>0</v>
       </c>
-    </row>
-    <row r="163" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="V162" t="s">
+        <v>346</v>
+      </c>
+      <c r="W162" t="s">
+        <v>347</v>
+      </c>
+    </row>
+    <row r="163" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A163">
         <v>48</v>
       </c>
@@ -12131,8 +13374,14 @@
       <c r="U163">
         <v>1</v>
       </c>
-    </row>
-    <row r="164" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="V163" t="s">
+        <v>350</v>
+      </c>
+      <c r="W163" t="s">
+        <v>350</v>
+      </c>
+    </row>
+    <row r="164" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A164">
         <v>48</v>
       </c>
@@ -12196,8 +13445,14 @@
       <c r="U164">
         <v>0</v>
       </c>
-    </row>
-    <row r="165" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="V164" t="s">
+        <v>350</v>
+      </c>
+      <c r="W164" t="s">
+        <v>350</v>
+      </c>
+    </row>
+    <row r="165" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A165">
         <v>48</v>
       </c>
@@ -12261,8 +13516,14 @@
       <c r="U165">
         <v>0</v>
       </c>
-    </row>
-    <row r="166" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="V165" t="s">
+        <v>346</v>
+      </c>
+      <c r="W165" t="s">
+        <v>347</v>
+      </c>
+    </row>
+    <row r="166" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A166">
         <v>48</v>
       </c>
@@ -12326,8 +13587,14 @@
       <c r="U166">
         <v>1</v>
       </c>
-    </row>
-    <row r="167" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="V166" t="s">
+        <v>346</v>
+      </c>
+      <c r="W166" t="s">
+        <v>347</v>
+      </c>
+    </row>
+    <row r="167" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A167">
         <v>48</v>
       </c>
@@ -12391,8 +13658,14 @@
       <c r="U167">
         <v>0</v>
       </c>
-    </row>
-    <row r="168" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="V167" t="s">
+        <v>357</v>
+      </c>
+      <c r="W167" t="s">
+        <v>358</v>
+      </c>
+    </row>
+    <row r="168" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A168">
         <v>4</v>
       </c>
@@ -12456,8 +13729,14 @@
       <c r="U168">
         <v>0</v>
       </c>
-    </row>
-    <row r="169" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="V168" t="s">
+        <v>410</v>
+      </c>
+      <c r="W168" t="s">
+        <v>411</v>
+      </c>
+    </row>
+    <row r="169" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A169">
         <v>4</v>
       </c>
@@ -12521,8 +13800,14 @@
       <c r="U169">
         <v>0</v>
       </c>
-    </row>
-    <row r="170" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="V169" t="s">
+        <v>359</v>
+      </c>
+      <c r="W169" t="s">
+        <v>360</v>
+      </c>
+    </row>
+    <row r="170" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A170">
         <v>4</v>
       </c>
@@ -12586,8 +13871,14 @@
       <c r="U170">
         <v>0</v>
       </c>
-    </row>
-    <row r="171" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="V170" t="s">
+        <v>412</v>
+      </c>
+      <c r="W170" t="s">
+        <v>413</v>
+      </c>
+    </row>
+    <row r="171" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A171">
         <v>50</v>
       </c>
@@ -12651,8 +13942,14 @@
       <c r="U171">
         <v>0</v>
       </c>
-    </row>
-    <row r="172" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="V171" t="s">
+        <v>414</v>
+      </c>
+      <c r="W171" t="s">
+        <v>415</v>
+      </c>
+    </row>
+    <row r="172" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A172">
         <v>50</v>
       </c>
@@ -12716,8 +14013,14 @@
       <c r="U172">
         <v>0</v>
       </c>
-    </row>
-    <row r="173" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="V172" t="s">
+        <v>346</v>
+      </c>
+      <c r="W172" t="s">
+        <v>347</v>
+      </c>
+    </row>
+    <row r="173" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A173">
         <v>50</v>
       </c>
@@ -12781,8 +14084,14 @@
       <c r="U173">
         <v>0</v>
       </c>
-    </row>
-    <row r="174" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="V173" t="s">
+        <v>350</v>
+      </c>
+      <c r="W173" t="s">
+        <v>350</v>
+      </c>
+    </row>
+    <row r="174" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A174">
         <v>50</v>
       </c>
@@ -12846,8 +14155,14 @@
       <c r="U174">
         <v>0</v>
       </c>
-    </row>
-    <row r="175" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="V174" t="s">
+        <v>346</v>
+      </c>
+      <c r="W174" t="s">
+        <v>347</v>
+      </c>
+    </row>
+    <row r="175" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A175">
         <v>51</v>
       </c>
@@ -12911,8 +14226,14 @@
       <c r="U175">
         <v>0</v>
       </c>
-    </row>
-    <row r="176" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="V175" t="s">
+        <v>348</v>
+      </c>
+      <c r="W175" t="s">
+        <v>349</v>
+      </c>
+    </row>
+    <row r="176" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A176">
         <v>51</v>
       </c>
@@ -12976,8 +14297,14 @@
       <c r="U176">
         <v>0</v>
       </c>
-    </row>
-    <row r="177" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="V176" t="s">
+        <v>346</v>
+      </c>
+      <c r="W176" t="s">
+        <v>347</v>
+      </c>
+    </row>
+    <row r="177" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A177">
         <v>51</v>
       </c>
@@ -13041,8 +14368,14 @@
       <c r="U177">
         <v>0</v>
       </c>
-    </row>
-    <row r="178" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="V177" t="s">
+        <v>346</v>
+      </c>
+      <c r="W177" t="s">
+        <v>347</v>
+      </c>
+    </row>
+    <row r="178" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A178">
         <v>51</v>
       </c>
@@ -13106,8 +14439,14 @@
       <c r="U178">
         <v>0</v>
       </c>
-    </row>
-    <row r="179" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="V178" t="s">
+        <v>353</v>
+      </c>
+      <c r="W178" t="s">
+        <v>354</v>
+      </c>
+    </row>
+    <row r="179" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A179">
         <v>51</v>
       </c>
@@ -13171,8 +14510,14 @@
       <c r="U179">
         <v>1</v>
       </c>
-    </row>
-    <row r="180" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="V179" t="s">
+        <v>346</v>
+      </c>
+      <c r="W179" t="s">
+        <v>347</v>
+      </c>
+    </row>
+    <row r="180" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A180">
         <v>51</v>
       </c>
@@ -13236,8 +14581,14 @@
       <c r="U180">
         <v>0</v>
       </c>
-    </row>
-    <row r="181" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="V180" t="s">
+        <v>416</v>
+      </c>
+      <c r="W180" t="s">
+        <v>417</v>
+      </c>
+    </row>
+    <row r="181" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A181">
         <v>52</v>
       </c>
@@ -13301,8 +14652,14 @@
       <c r="U181">
         <v>0</v>
       </c>
-    </row>
-    <row r="182" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="V181" t="s">
+        <v>376</v>
+      </c>
+      <c r="W181" t="s">
+        <v>377</v>
+      </c>
+    </row>
+    <row r="182" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A182">
         <v>53</v>
       </c>
@@ -13366,8 +14723,14 @@
       <c r="U182">
         <v>0</v>
       </c>
-    </row>
-    <row r="183" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="V182" t="s">
+        <v>400</v>
+      </c>
+      <c r="W182" t="s">
+        <v>401</v>
+      </c>
+    </row>
+    <row r="183" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A183">
         <v>53</v>
       </c>
@@ -13431,8 +14794,14 @@
       <c r="U183">
         <v>0</v>
       </c>
-    </row>
-    <row r="184" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="V183" t="s">
+        <v>346</v>
+      </c>
+      <c r="W183" t="s">
+        <v>347</v>
+      </c>
+    </row>
+    <row r="184" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A184">
         <v>53</v>
       </c>
@@ -13496,8 +14865,14 @@
       <c r="U184">
         <v>0</v>
       </c>
-    </row>
-    <row r="185" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="V184" t="s">
+        <v>346</v>
+      </c>
+      <c r="W184" t="s">
+        <v>347</v>
+      </c>
+    </row>
+    <row r="185" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A185">
         <v>5</v>
       </c>
@@ -13561,8 +14936,14 @@
       <c r="U185">
         <v>1</v>
       </c>
-    </row>
-    <row r="186" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="V185" t="s">
+        <v>369</v>
+      </c>
+      <c r="W185" t="s">
+        <v>368</v>
+      </c>
+    </row>
+    <row r="186" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A186">
         <v>5</v>
       </c>
@@ -13626,8 +15007,14 @@
       <c r="U186">
         <v>2</v>
       </c>
-    </row>
-    <row r="187" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="V186" t="s">
+        <v>355</v>
+      </c>
+      <c r="W186" t="s">
+        <v>356</v>
+      </c>
+    </row>
+    <row r="187" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A187">
         <v>65</v>
       </c>
@@ -13691,8 +15078,14 @@
       <c r="U187">
         <v>0</v>
       </c>
-    </row>
-    <row r="188" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="V187" t="s">
+        <v>346</v>
+      </c>
+      <c r="W187" t="s">
+        <v>347</v>
+      </c>
+    </row>
+    <row r="188" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A188">
         <v>6</v>
       </c>
@@ -13756,8 +15149,14 @@
       <c r="U188">
         <v>0</v>
       </c>
-    </row>
-    <row r="189" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="V188" t="s">
+        <v>357</v>
+      </c>
+      <c r="W188" t="s">
+        <v>358</v>
+      </c>
+    </row>
+    <row r="189" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A189">
         <v>6</v>
       </c>
@@ -13821,8 +15220,14 @@
       <c r="U189">
         <v>0</v>
       </c>
-    </row>
-    <row r="190" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="V189" t="s">
+        <v>386</v>
+      </c>
+      <c r="W189" t="s">
+        <v>387</v>
+      </c>
+    </row>
+    <row r="190" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A190">
         <v>6</v>
       </c>
@@ -13886,8 +15291,14 @@
       <c r="U190">
         <v>1</v>
       </c>
-    </row>
-    <row r="191" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="V190" t="s">
+        <v>346</v>
+      </c>
+      <c r="W190" t="s">
+        <v>347</v>
+      </c>
+    </row>
+    <row r="191" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A191">
         <v>6</v>
       </c>
@@ -13951,8 +15362,14 @@
       <c r="U191">
         <v>0</v>
       </c>
-    </row>
-    <row r="192" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="V191" t="s">
+        <v>359</v>
+      </c>
+      <c r="W191" t="s">
+        <v>360</v>
+      </c>
+    </row>
+    <row r="192" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A192">
         <v>6</v>
       </c>
@@ -14016,8 +15433,14 @@
       <c r="U192">
         <v>0</v>
       </c>
-    </row>
-    <row r="193" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="V192" t="s">
+        <v>346</v>
+      </c>
+      <c r="W192" t="s">
+        <v>347</v>
+      </c>
+    </row>
+    <row r="193" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A193">
         <v>6</v>
       </c>
@@ -14081,8 +15504,14 @@
       <c r="U193">
         <v>0</v>
       </c>
-    </row>
-    <row r="194" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="V193" t="s">
+        <v>346</v>
+      </c>
+      <c r="W193" t="s">
+        <v>347</v>
+      </c>
+    </row>
+    <row r="194" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A194">
         <v>6</v>
       </c>
@@ -14146,8 +15575,14 @@
       <c r="U194">
         <v>0</v>
       </c>
-    </row>
-    <row r="195" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="V194" t="s">
+        <v>346</v>
+      </c>
+      <c r="W194" t="s">
+        <v>347</v>
+      </c>
+    </row>
+    <row r="195" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A195">
         <v>6</v>
       </c>
@@ -14211,8 +15646,14 @@
       <c r="U195">
         <v>0</v>
       </c>
-    </row>
-    <row r="196" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="V195" t="s">
+        <v>346</v>
+      </c>
+      <c r="W195" t="s">
+        <v>347</v>
+      </c>
+    </row>
+    <row r="196" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A196">
         <v>7</v>
       </c>
@@ -14276,8 +15717,14 @@
       <c r="U196">
         <v>0</v>
       </c>
-    </row>
-    <row r="197" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="V196" t="s">
+        <v>350</v>
+      </c>
+      <c r="W196" t="s">
+        <v>350</v>
+      </c>
+    </row>
+    <row r="197" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A197">
         <v>7</v>
       </c>
@@ -14341,8 +15788,14 @@
       <c r="U197">
         <v>0</v>
       </c>
-    </row>
-    <row r="198" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="V197" t="s">
+        <v>350</v>
+      </c>
+      <c r="W197" t="s">
+        <v>350</v>
+      </c>
+    </row>
+    <row r="198" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A198">
         <v>7</v>
       </c>
@@ -14406,8 +15859,14 @@
       <c r="U198">
         <v>0</v>
       </c>
-    </row>
-    <row r="199" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="V198" t="s">
+        <v>350</v>
+      </c>
+      <c r="W198" t="s">
+        <v>350</v>
+      </c>
+    </row>
+    <row r="199" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A199">
         <v>7</v>
       </c>
@@ -14471,8 +15930,14 @@
       <c r="U199">
         <v>1</v>
       </c>
-    </row>
-    <row r="200" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="V199" t="s">
+        <v>392</v>
+      </c>
+      <c r="W199" t="s">
+        <v>393</v>
+      </c>
+    </row>
+    <row r="200" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A200">
         <v>7</v>
       </c>
@@ -14536,8 +16001,14 @@
       <c r="U200">
         <v>0</v>
       </c>
-    </row>
-    <row r="201" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="V200" t="s">
+        <v>350</v>
+      </c>
+      <c r="W200" t="s">
+        <v>350</v>
+      </c>
+    </row>
+    <row r="201" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A201">
         <v>7</v>
       </c>
@@ -14601,8 +16072,14 @@
       <c r="U201">
         <v>0</v>
       </c>
-    </row>
-    <row r="202" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="V201" t="s">
+        <v>418</v>
+      </c>
+      <c r="W201" t="s">
+        <v>419</v>
+      </c>
+    </row>
+    <row r="202" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A202">
         <v>7</v>
       </c>
@@ -14666,8 +16143,14 @@
       <c r="U202">
         <v>0</v>
       </c>
-    </row>
-    <row r="203" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="V202" t="s">
+        <v>350</v>
+      </c>
+      <c r="W202" t="s">
+        <v>350</v>
+      </c>
+    </row>
+    <row r="203" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A203">
         <v>7</v>
       </c>
@@ -14731,8 +16214,14 @@
       <c r="U203">
         <v>0</v>
       </c>
-    </row>
-    <row r="204" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="V203" t="s">
+        <v>350</v>
+      </c>
+      <c r="W203" t="s">
+        <v>350</v>
+      </c>
+    </row>
+    <row r="204" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A204">
         <v>8</v>
       </c>
@@ -14796,8 +16285,14 @@
       <c r="U204">
         <v>0</v>
       </c>
-    </row>
-    <row r="205" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="V204" t="s">
+        <v>350</v>
+      </c>
+      <c r="W204" t="s">
+        <v>350</v>
+      </c>
+    </row>
+    <row r="205" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A205">
         <v>8</v>
       </c>
@@ -14861,8 +16356,14 @@
       <c r="U205">
         <v>0</v>
       </c>
-    </row>
-    <row r="206" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="V205" t="s">
+        <v>350</v>
+      </c>
+      <c r="W205" t="s">
+        <v>350</v>
+      </c>
+    </row>
+    <row r="206" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A206">
         <v>8</v>
       </c>
@@ -14926,8 +16427,14 @@
       <c r="U206">
         <v>0</v>
       </c>
-    </row>
-    <row r="207" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="V206" t="s">
+        <v>390</v>
+      </c>
+      <c r="W206" t="s">
+        <v>391</v>
+      </c>
+    </row>
+    <row r="207" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A207">
         <v>8</v>
       </c>
@@ -14991,8 +16498,14 @@
       <c r="U207">
         <v>2</v>
       </c>
-    </row>
-    <row r="208" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="V207" t="s">
+        <v>420</v>
+      </c>
+      <c r="W207" t="s">
+        <v>421</v>
+      </c>
+    </row>
+    <row r="208" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A208">
         <v>9</v>
       </c>
@@ -15056,8 +16569,14 @@
       <c r="U208">
         <v>0</v>
       </c>
-    </row>
-    <row r="209" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="V208" t="s">
+        <v>422</v>
+      </c>
+      <c r="W208" t="s">
+        <v>423</v>
+      </c>
+    </row>
+    <row r="209" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A209">
         <v>9</v>
       </c>
@@ -15121,8 +16640,14 @@
       <c r="U209">
         <v>0</v>
       </c>
-    </row>
-    <row r="210" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="V209" t="s">
+        <v>346</v>
+      </c>
+      <c r="W209" t="s">
+        <v>347</v>
+      </c>
+    </row>
+    <row r="210" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A210">
         <v>9</v>
       </c>
@@ -15186,8 +16711,14 @@
       <c r="U210">
         <v>0</v>
       </c>
-    </row>
-    <row r="211" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="V210" t="s">
+        <v>392</v>
+      </c>
+      <c r="W210" t="s">
+        <v>393</v>
+      </c>
+    </row>
+    <row r="211" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A211">
         <v>9</v>
       </c>
@@ -15251,8 +16782,14 @@
       <c r="U211">
         <v>0</v>
       </c>
-    </row>
-    <row r="212" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="V211" t="s">
+        <v>424</v>
+      </c>
+      <c r="W211" t="s">
+        <v>425</v>
+      </c>
+    </row>
+    <row r="212" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A212">
         <v>9</v>
       </c>
@@ -15316,8 +16853,14 @@
       <c r="U212">
         <v>0</v>
       </c>
-    </row>
-    <row r="213" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="V212" t="s">
+        <v>346</v>
+      </c>
+      <c r="W212" t="s">
+        <v>347</v>
+      </c>
+    </row>
+    <row r="213" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A213">
         <v>9</v>
       </c>
@@ -15380,6 +16923,12 @@
       </c>
       <c r="U213">
         <v>0</v>
+      </c>
+      <c r="V213" t="s">
+        <v>426</v>
+      </c>
+      <c r="W213" t="s">
+        <v>427</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Meias quitando planificacion 0
</commit_message>
<xml_diff>
--- a/datosNivelesMedias.xlsx
+++ b/datosNivelesMedias.xlsx
@@ -1,20 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\hlocal\C_TFG\Datos\Mision Colombia-20260209T150018Z-3-001\jsonToCsv_TFG\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2DCD2B5A-8BEC-4304-A84B-A8DF60E494D5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{91964B7D-C697-43C6-82C1-94F7295EDC54}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
     <sheet name="Hoja1" sheetId="2" r:id="rId2"/>
+    <sheet name="Hoja2" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -56,7 +57,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="579" uniqueCount="351">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="619" uniqueCount="351">
   <si>
     <t>ID</t>
   </si>
@@ -17329,4 +17330,627 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E7E06012-538D-4879-B4D7-76AF65331837}">
+  <dimension ref="A1:AF9"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetData>
+    <row r="1" spans="1:32" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>307</v>
+      </c>
+      <c r="B1" t="s">
+        <v>308</v>
+      </c>
+      <c r="C1" t="s">
+        <v>309</v>
+      </c>
+      <c r="D1" t="s">
+        <v>310</v>
+      </c>
+      <c r="E1" t="s">
+        <v>311</v>
+      </c>
+      <c r="F1" t="s">
+        <v>312</v>
+      </c>
+      <c r="G1" t="s">
+        <v>313</v>
+      </c>
+      <c r="H1" t="s">
+        <v>314</v>
+      </c>
+      <c r="I1" t="s">
+        <v>315</v>
+      </c>
+      <c r="J1" t="s">
+        <v>316</v>
+      </c>
+      <c r="K1" t="s">
+        <v>317</v>
+      </c>
+      <c r="L1" t="s">
+        <v>318</v>
+      </c>
+      <c r="M1" t="s">
+        <v>319</v>
+      </c>
+      <c r="N1" t="s">
+        <v>320</v>
+      </c>
+      <c r="O1" t="s">
+        <v>321</v>
+      </c>
+      <c r="P1" t="s">
+        <v>322</v>
+      </c>
+      <c r="Q1" t="s">
+        <v>323</v>
+      </c>
+      <c r="R1" t="s">
+        <v>324</v>
+      </c>
+      <c r="S1" t="s">
+        <v>325</v>
+      </c>
+      <c r="T1" t="s">
+        <v>326</v>
+      </c>
+      <c r="U1" t="s">
+        <v>327</v>
+      </c>
+      <c r="V1" t="s">
+        <v>328</v>
+      </c>
+      <c r="W1" t="s">
+        <v>329</v>
+      </c>
+      <c r="X1" t="s">
+        <v>330</v>
+      </c>
+      <c r="Y1" t="s">
+        <v>331</v>
+      </c>
+      <c r="Z1" t="s">
+        <v>332</v>
+      </c>
+      <c r="AA1" t="s">
+        <v>333</v>
+      </c>
+      <c r="AB1" t="s">
+        <v>334</v>
+      </c>
+      <c r="AC1" t="s">
+        <v>343</v>
+      </c>
+      <c r="AD1" t="s">
+        <v>344</v>
+      </c>
+      <c r="AE1" t="s">
+        <v>345</v>
+      </c>
+      <c r="AF1" t="s">
+        <v>346</v>
+      </c>
+    </row>
+    <row r="2" spans="1:32" x14ac:dyDescent="0.3">
+      <c r="A2">
+        <v>1</v>
+      </c>
+      <c r="B2">
+        <f>COUNTIFS(dataNiveles[Nivel],A2,dataNiveles[Pasos planificados],"&gt;0")</f>
+        <v>70</v>
+      </c>
+      <c r="C2">
+        <f>AVERAGEIFS(dataNiveles[Pasos planificados],dataNiveles[Nivel],A2,dataNiveles[Pasos planificados],"&gt;0")</f>
+        <v>9.8714285714285719</v>
+      </c>
+      <c r="D2" cm="1">
+        <f t="array" ref="D2">_xlfn.STDEV.P(IF((dataNiveles[Nivel]=A2)*(dataNiveles[Pasos planificados]&lt;&gt;0),dataNiveles[Pasos planificados]))</f>
+        <v>7.6865772218689834</v>
+      </c>
+      <c r="E2">
+        <f>AVERAGEIFS(dataNiveles[Pasos ejecutados],dataNiveles[Nivel],A2,dataNiveles[Pasos planificados],"&gt;0")</f>
+        <v>8.0285714285714285</v>
+      </c>
+      <c r="F2" cm="1">
+        <f t="array" ref="F2">_xlfn.STDEV.P(IF((dataNiveles[Nivel]=A2)*(dataNiveles[Pasos planificados]&lt;&gt;0),dataNiveles[Pasos ejecutados]))</f>
+        <v>5.8357798562499124</v>
+      </c>
+      <c r="G2">
+        <f>AVERAGEIFS(dataNiveles[Errores ejecucion],dataNiveles[Nivel],A2,dataNiveles[Pasos planificados],"&gt;0")</f>
+        <v>1.8428571428571427</v>
+      </c>
+      <c r="H2" cm="1">
+        <f t="array" ref="H2">_xlfn.STDEV.P(IF((dataNiveles[Nivel]=A2)*(dataNiveles[Pasos planificados]&lt;&gt;0),dataNiveles[Errores ejecucion]))</f>
+        <v>2.6866639658331151</v>
+      </c>
+      <c r="I2">
+        <f>AVERAGEIFS(dataNiveles[Num dormir planificado],dataNiveles[Nivel],A2,dataNiveles[Pasos planificados],"&gt;0")</f>
+        <v>4.7714285714285714</v>
+      </c>
+      <c r="J2" cm="1">
+        <f t="array" ref="J2">_xlfn.STDEV.P(IF((dataNiveles[Nivel]=A2)*(dataNiveles[Pasos planificados]&lt;&gt;0),dataNiveles[Num dormir planificado]))</f>
+        <v>3.4524170769866998</v>
+      </c>
+      <c r="K2">
+        <f>AVERAGEIFS(dataNiveles[Correctos dormir],dataNiveles[Nivel],A2,dataNiveles[Pasos planificados],"&gt;0")</f>
+        <v>4.4714285714285715</v>
+      </c>
+      <c r="L2" cm="1">
+        <f t="array" ref="L2">_xlfn.STDEV.P(IF((dataNiveles[Nivel]=A2)*(dataNiveles[Pasos planificados]&lt;&gt;0),dataNiveles[Correctos dormir]))</f>
+        <v>3.1745480153938161</v>
+      </c>
+      <c r="M2">
+        <f>AVERAGEIFS(dataNiveles[Errores dormir],dataNiveles[Nivel],A2,dataNiveles[Pasos planificados],"&gt;0")</f>
+        <v>0.3</v>
+      </c>
+      <c r="N2" cm="1">
+        <f t="array" ref="N2">_xlfn.STDEV.P(IF((dataNiveles[Nivel]=A2)*(dataNiveles[Pasos planificados]&lt;&gt;0),dataNiveles[Errores dormir]))</f>
+        <v>0.91573545774499121</v>
+      </c>
+      <c r="O2">
+        <f>AVERAGEIFS(dataNiveles[Num ubicacion planificado],dataNiveles[Nivel],A2,dataNiveles[Pasos planificados],"&gt;0")</f>
+        <v>5.0999999999999996</v>
+      </c>
+      <c r="P2" cm="1">
+        <f t="array" ref="P2">_xlfn.STDEV.P(IF((dataNiveles[Nivel]=A2)*(dataNiveles[Pasos planificados]&lt;&gt;0),dataNiveles[Num ubicacion planificado]))</f>
+        <v>4.9602707299386104</v>
+      </c>
+      <c r="Q2">
+        <f>AVERAGEIFS(dataNiveles[Correctos ubicacion],dataNiveles[Nivel],A2,dataNiveles[Pasos planificados],"&gt;0")</f>
+        <v>3.5571428571428569</v>
+      </c>
+      <c r="R2" cm="1">
+        <f t="array" ref="R2">_xlfn.STDEV.P(IF((dataNiveles[Nivel]=A2)*(dataNiveles[Pasos planificados]&lt;&gt;0),dataNiveles[Correctos ubicacion]))</f>
+        <v>3.2716780940398777</v>
+      </c>
+      <c r="S2">
+        <f>AVERAGEIFS(dataNiveles[Errores ubicacion],dataNiveles[Nivel],A2,dataNiveles[Pasos planificados],"&gt;0")</f>
+        <v>1.5428571428571429</v>
+      </c>
+      <c r="T2" cm="1">
+        <f t="array" ref="T2">_xlfn.STDEV.P(IF((dataNiveles[Nivel]=A2)*(dataNiveles[Pasos planificados]&lt;&gt;0),dataNiveles[Errores ubicacion]))</f>
+        <v>2.4005101498622823</v>
+      </c>
+      <c r="U2">
+        <f>AVERAGEIFS(dataNiveles[Paradas posibles],dataNiveles[Nivel],A2,dataNiveles[Pasos planificados],"&gt;0")</f>
+        <v>9.6857142857142851</v>
+      </c>
+      <c r="V2" cm="1">
+        <f t="array" ref="V2">_xlfn.STDEV.P(IF((dataNiveles[Nivel]=A2)*(dataNiveles[Pasos planificados]&lt;&gt;0),dataNiveles[Paradas posibles]))</f>
+        <v>6.6150107593970526</v>
+      </c>
+      <c r="W2">
+        <f>AVERAGEIFS(dataNiveles[Paradas realizadas],dataNiveles[Nivel],A2,dataNiveles[Pasos planificados],"&gt;0")</f>
+        <v>7.2142857142857144</v>
+      </c>
+      <c r="X2" cm="1">
+        <f t="array" ref="X2">_xlfn.STDEV.P(IF((dataNiveles[Nivel]=A2)*(dataNiveles[Pasos planificados]&lt;&gt;0),dataNiveles[Paradas realizadas]))</f>
+        <v>5.3556188308378045</v>
+      </c>
+      <c r="Y2">
+        <f>AVERAGEIFS(dataNiveles[Errores parada por tiempo excedido],dataNiveles[Nivel],A2,dataNiveles[Pasos planificados],"&gt;0")</f>
+        <v>0.14285714285714285</v>
+      </c>
+      <c r="Z2" cm="1">
+        <f t="array" ref="Z2">_xlfn.STDEV.P(IF((dataNiveles[Nivel]=A2)*(dataNiveles[Pasos planificados]&lt;&gt;0),dataNiveles[Errores parada por tiempo excedido]))</f>
+        <v>0.4237827706911807</v>
+      </c>
+      <c r="AA2">
+        <f>AVERAGEIFS(dataNiveles[Num errores por tiempo excedido],dataNiveles[Nivel],A2,dataNiveles[Pasos planificados],"&gt;0")</f>
+        <v>0.14285714285714285</v>
+      </c>
+      <c r="AB2" cm="1">
+        <f t="array" ref="AB2">_xlfn.STDEV.P(IF((dataNiveles[Nivel]=A2)*(dataNiveles[Pasos planificados]&lt;&gt;0),dataNiveles[Num errores por tiempo excedido]))</f>
+        <v>0.4237827706911807</v>
+      </c>
+      <c r="AC2">
+        <f>AVERAGEIFS(dataNiveles[% Aciertos],dataNiveles[Nivel],A2,dataNiveles[Pasos planificados],"&gt;0")</f>
+        <v>85.815476031893851</v>
+      </c>
+      <c r="AD2" cm="1">
+        <f t="array" ref="AD2">_xlfn.STDEV.P(IF((dataNiveles[Nivel]=A2)*(dataNiveles[Pasos planificados]&lt;&gt;0),dataNiveles[% Aciertos]))</f>
+        <v>15.269100509855848</v>
+      </c>
+      <c r="AE2">
+        <f>AVERAGEIFS(dataNiveles[% Mal],dataNiveles[Nivel],A2,dataNiveles[Pasos planificados],"&gt;0")</f>
+        <v>14.184523968106102</v>
+      </c>
+      <c r="AF2" cm="1">
+        <f t="array" ref="AF2">_xlfn.STDEV.P(IF((dataNiveles[Nivel]=A2)*(dataNiveles[Pasos planificados]&lt;&gt;0),dataNiveles[% Mal]))</f>
+        <v>15.269100509855752</v>
+      </c>
+    </row>
+    <row r="3" spans="1:32" x14ac:dyDescent="0.3">
+      <c r="A3">
+        <v>2</v>
+      </c>
+      <c r="B3">
+        <f>COUNTIFS(dataNiveles[Nivel],A3,dataNiveles[Pasos planificados],"&gt;0")</f>
+        <v>54</v>
+      </c>
+      <c r="C3">
+        <f>AVERAGEIFS(dataNiveles[Pasos planificados],dataNiveles[Nivel],A3,dataNiveles[Pasos planificados],"&gt;0")</f>
+        <v>7.6111111111111107</v>
+      </c>
+      <c r="D3" cm="1">
+        <f t="array" ref="D3">_xlfn.STDEV.P(IF((dataNiveles[Nivel]=A3)*(dataNiveles[Pasos planificados]&lt;&gt;0),dataNiveles[Pasos planificados]))</f>
+        <v>6.5839779337493809</v>
+      </c>
+      <c r="E3">
+        <f>AVERAGEIFS(dataNiveles[Pasos ejecutados],dataNiveles[Nivel],A3,dataNiveles[Pasos planificados],"&gt;0")</f>
+        <v>6.6296296296296298</v>
+      </c>
+      <c r="F3" cm="1">
+        <f t="array" ref="F3">_xlfn.STDEV.P(IF((dataNiveles[Nivel]=A3)*(dataNiveles[Pasos planificados]&lt;&gt;0),dataNiveles[Pasos ejecutados]))</f>
+        <v>5.6578241344972771</v>
+      </c>
+      <c r="G3">
+        <f>AVERAGEIFS(dataNiveles[Errores ejecucion],dataNiveles[Nivel],A3,dataNiveles[Pasos planificados],"&gt;0")</f>
+        <v>0.98148148148148151</v>
+      </c>
+      <c r="H3" cm="1">
+        <f t="array" ref="H3">_xlfn.STDEV.P(IF((dataNiveles[Nivel]=A3)*(dataNiveles[Pasos planificados]&lt;&gt;0),dataNiveles[Errores ejecucion]))</f>
+        <v>1.5927002547588534</v>
+      </c>
+      <c r="I3">
+        <f>AVERAGEIFS(dataNiveles[Num dormir planificado],dataNiveles[Nivel],A3,dataNiveles[Pasos planificados],"&gt;0")</f>
+        <v>4.1481481481481479</v>
+      </c>
+      <c r="J3" cm="1">
+        <f t="array" ref="J3">_xlfn.STDEV.P(IF((dataNiveles[Nivel]=A3)*(dataNiveles[Pasos planificados]&lt;&gt;0),dataNiveles[Num dormir planificado]))</f>
+        <v>3.5559413370958386</v>
+      </c>
+      <c r="K3">
+        <f>AVERAGEIFS(dataNiveles[Correctos dormir],dataNiveles[Nivel],A3,dataNiveles[Pasos planificados],"&gt;0")</f>
+        <v>3.9074074074074074</v>
+      </c>
+      <c r="L3" cm="1">
+        <f t="array" ref="L3">_xlfn.STDEV.P(IF((dataNiveles[Nivel]=A3)*(dataNiveles[Pasos planificados]&lt;&gt;0),dataNiveles[Correctos dormir]))</f>
+        <v>3.4762075893694231</v>
+      </c>
+      <c r="M3">
+        <f>AVERAGEIFS(dataNiveles[Errores dormir],dataNiveles[Nivel],A3,dataNiveles[Pasos planificados],"&gt;0")</f>
+        <v>0.24074074074074073</v>
+      </c>
+      <c r="N3" cm="1">
+        <f t="array" ref="N3">_xlfn.STDEV.P(IF((dataNiveles[Nivel]=A3)*(dataNiveles[Pasos planificados]&lt;&gt;0),dataNiveles[Errores dormir]))</f>
+        <v>0.66486381744504597</v>
+      </c>
+      <c r="O3">
+        <f>AVERAGEIFS(dataNiveles[Num ubicacion planificado],dataNiveles[Nivel],A3,dataNiveles[Pasos planificados],"&gt;0")</f>
+        <v>3.4629629629629628</v>
+      </c>
+      <c r="P3" cm="1">
+        <f t="array" ref="P3">_xlfn.STDEV.P(IF((dataNiveles[Nivel]=A3)*(dataNiveles[Pasos planificados]&lt;&gt;0),dataNiveles[Num ubicacion planificado]))</f>
+        <v>3.2869718303391458</v>
+      </c>
+      <c r="Q3">
+        <f>AVERAGEIFS(dataNiveles[Correctos ubicacion],dataNiveles[Nivel],A3,dataNiveles[Pasos planificados],"&gt;0")</f>
+        <v>2.7222222222222223</v>
+      </c>
+      <c r="R3" cm="1">
+        <f t="array" ref="R3">_xlfn.STDEV.P(IF((dataNiveles[Nivel]=A3)*(dataNiveles[Pasos planificados]&lt;&gt;0),dataNiveles[Correctos ubicacion]))</f>
+        <v>2.5633937766798507</v>
+      </c>
+      <c r="S3">
+        <f>AVERAGEIFS(dataNiveles[Errores ubicacion],dataNiveles[Nivel],A3,dataNiveles[Pasos planificados],"&gt;0")</f>
+        <v>0.7407407407407407</v>
+      </c>
+      <c r="T3" cm="1">
+        <f t="array" ref="T3">_xlfn.STDEV.P(IF((dataNiveles[Nivel]=A3)*(dataNiveles[Pasos planificados]&lt;&gt;0),dataNiveles[Errores ubicacion]))</f>
+        <v>1.2792530399385587</v>
+      </c>
+      <c r="U3">
+        <f>AVERAGEIFS(dataNiveles[Paradas posibles],dataNiveles[Nivel],A3,dataNiveles[Pasos planificados],"&gt;0")</f>
+        <v>8.8518518518518512</v>
+      </c>
+      <c r="V3" cm="1">
+        <f t="array" ref="V3">_xlfn.STDEV.P(IF((dataNiveles[Nivel]=A3)*(dataNiveles[Pasos planificados]&lt;&gt;0),dataNiveles[Paradas posibles]))</f>
+        <v>9.1841397254490111</v>
+      </c>
+      <c r="W3">
+        <f>AVERAGEIFS(dataNiveles[Paradas realizadas],dataNiveles[Nivel],A3,dataNiveles[Pasos planificados],"&gt;0")</f>
+        <v>5.6481481481481479</v>
+      </c>
+      <c r="X3" cm="1">
+        <f t="array" ref="X3">_xlfn.STDEV.P(IF((dataNiveles[Nivel]=A3)*(dataNiveles[Pasos planificados]&lt;&gt;0),dataNiveles[Paradas realizadas]))</f>
+        <v>6.4439388903446755</v>
+      </c>
+      <c r="Y3">
+        <f>AVERAGEIFS(dataNiveles[Errores parada por tiempo excedido],dataNiveles[Nivel],A3,dataNiveles[Pasos planificados],"&gt;0")</f>
+        <v>0.81481481481481477</v>
+      </c>
+      <c r="Z3" cm="1">
+        <f t="array" ref="Z3">_xlfn.STDEV.P(IF((dataNiveles[Nivel]=A3)*(dataNiveles[Pasos planificados]&lt;&gt;0),dataNiveles[Errores parada por tiempo excedido]))</f>
+        <v>1.1233889546743037</v>
+      </c>
+      <c r="AA3">
+        <f>AVERAGEIFS(dataNiveles[Num errores por tiempo excedido],dataNiveles[Nivel],A3,dataNiveles[Pasos planificados],"&gt;0")</f>
+        <v>1</v>
+      </c>
+      <c r="AB3" cm="1">
+        <f t="array" ref="AB3">_xlfn.STDEV.P(IF((dataNiveles[Nivel]=A3)*(dataNiveles[Pasos planificados]&lt;&gt;0),dataNiveles[Num errores por tiempo excedido]))</f>
+        <v>1.4529663145135578</v>
+      </c>
+      <c r="AC3">
+        <f>AVERAGEIFS(dataNiveles[% Aciertos],dataNiveles[Nivel],A3,dataNiveles[Pasos planificados],"&gt;0")</f>
+        <v>87.697510822510807</v>
+      </c>
+      <c r="AD3" cm="1">
+        <f t="array" ref="AD3">_xlfn.STDEV.P(IF((dataNiveles[Nivel]=A3)*(dataNiveles[Pasos planificados]&lt;&gt;0),dataNiveles[% Aciertos]))</f>
+        <v>21.073686270495209</v>
+      </c>
+      <c r="AE3">
+        <f>AVERAGEIFS(dataNiveles[% Mal],dataNiveles[Nivel],A3,dataNiveles[Pasos planificados],"&gt;0")</f>
+        <v>12.302489177489166</v>
+      </c>
+      <c r="AF3" cm="1">
+        <f t="array" ref="AF3">_xlfn.STDEV.P(IF((dataNiveles[Nivel]=A3)*(dataNiveles[Pasos planificados]&lt;&gt;0),dataNiveles[% Mal]))</f>
+        <v>21.073686270495212</v>
+      </c>
+    </row>
+    <row r="4" spans="1:32" x14ac:dyDescent="0.3">
+      <c r="A4">
+        <v>3</v>
+      </c>
+      <c r="B4">
+        <f>COUNTIFS(dataNiveles[Nivel],A4,dataNiveles[Pasos planificados],"&gt;0")</f>
+        <v>42</v>
+      </c>
+      <c r="C4">
+        <f>AVERAGEIFS(dataNiveles[Pasos planificados],dataNiveles[Nivel],A4,dataNiveles[Pasos planificados],"&gt;0")</f>
+        <v>9.9285714285714288</v>
+      </c>
+      <c r="D4" cm="1">
+        <f t="array" ref="D4">_xlfn.STDEV.P(IF((dataNiveles[Nivel]=A4)*(dataNiveles[Pasos planificados]&lt;&gt;0),dataNiveles[Pasos planificados]))</f>
+        <v>8.7488580401560245</v>
+      </c>
+      <c r="E4">
+        <f>AVERAGEIFS(dataNiveles[Pasos ejecutados],dataNiveles[Nivel],A4,dataNiveles[Pasos planificados],"&gt;0")</f>
+        <v>8.2142857142857135</v>
+      </c>
+      <c r="F4" cm="1">
+        <f t="array" ref="F4">_xlfn.STDEV.P(IF((dataNiveles[Nivel]=A4)*(dataNiveles[Pasos planificados]&lt;&gt;0),dataNiveles[Pasos ejecutados]))</f>
+        <v>7.0661355852292802</v>
+      </c>
+      <c r="G4">
+        <f>AVERAGEIFS(dataNiveles[Errores ejecucion],dataNiveles[Nivel],A4,dataNiveles[Pasos planificados],"&gt;0")</f>
+        <v>1.7142857142857142</v>
+      </c>
+      <c r="H4" cm="1">
+        <f t="array" ref="H4">_xlfn.STDEV.P(IF((dataNiveles[Nivel]=A4)*(dataNiveles[Pasos planificados]&lt;&gt;0),dataNiveles[Errores ejecucion]))</f>
+        <v>2.1743714393963569</v>
+      </c>
+      <c r="I4">
+        <f>AVERAGEIFS(dataNiveles[Num dormir planificado],dataNiveles[Nivel],A4,dataNiveles[Pasos planificados],"&gt;0")</f>
+        <v>4.2857142857142856</v>
+      </c>
+      <c r="J4" cm="1">
+        <f t="array" ref="J4">_xlfn.STDEV.P(IF((dataNiveles[Nivel]=A4)*(dataNiveles[Pasos planificados]&lt;&gt;0),dataNiveles[Num dormir planificado]))</f>
+        <v>3.231435729014009</v>
+      </c>
+      <c r="K4">
+        <f>AVERAGEIFS(dataNiveles[Correctos dormir],dataNiveles[Nivel],A4,dataNiveles[Pasos planificados],"&gt;0")</f>
+        <v>4.1904761904761907</v>
+      </c>
+      <c r="L4" cm="1">
+        <f t="array" ref="L4">_xlfn.STDEV.P(IF((dataNiveles[Nivel]=A4)*(dataNiveles[Pasos planificados]&lt;&gt;0),dataNiveles[Correctos dormir]))</f>
+        <v>3.1715858676850881</v>
+      </c>
+      <c r="M4">
+        <f>AVERAGEIFS(dataNiveles[Errores dormir],dataNiveles[Nivel],A4,dataNiveles[Pasos planificados],"&gt;0")</f>
+        <v>9.5238095238095233E-2</v>
+      </c>
+      <c r="N4" cm="1">
+        <f t="array" ref="N4">_xlfn.STDEV.P(IF((dataNiveles[Nivel]=A4)*(dataNiveles[Pasos planificados]&lt;&gt;0),dataNiveles[Errores dormir]))</f>
+        <v>0.29354352395090366</v>
+      </c>
+      <c r="O4">
+        <f>AVERAGEIFS(dataNiveles[Num ubicacion planificado],dataNiveles[Nivel],A4,dataNiveles[Pasos planificados],"&gt;0")</f>
+        <v>5.6428571428571432</v>
+      </c>
+      <c r="P4" cm="1">
+        <f t="array" ref="P4">_xlfn.STDEV.P(IF((dataNiveles[Nivel]=A4)*(dataNiveles[Pasos planificados]&lt;&gt;0),dataNiveles[Num ubicacion planificado]))</f>
+        <v>6.0781475427156595</v>
+      </c>
+      <c r="Q4">
+        <f>AVERAGEIFS(dataNiveles[Correctos ubicacion],dataNiveles[Nivel],A4,dataNiveles[Pasos planificados],"&gt;0")</f>
+        <v>4.0238095238095237</v>
+      </c>
+      <c r="R4" cm="1">
+        <f t="array" ref="R4">_xlfn.STDEV.P(IF((dataNiveles[Nivel]=A4)*(dataNiveles[Pasos planificados]&lt;&gt;0),dataNiveles[Correctos ubicacion]))</f>
+        <v>4.7131431996982309</v>
+      </c>
+      <c r="S4">
+        <f>AVERAGEIFS(dataNiveles[Errores ubicacion],dataNiveles[Nivel],A4,dataNiveles[Pasos planificados],"&gt;0")</f>
+        <v>1.6190476190476191</v>
+      </c>
+      <c r="T4" cm="1">
+        <f t="array" ref="T4">_xlfn.STDEV.P(IF((dataNiveles[Nivel]=A4)*(dataNiveles[Pasos planificados]&lt;&gt;0),dataNiveles[Errores ubicacion]))</f>
+        <v>2.0581126461880292</v>
+      </c>
+      <c r="U4">
+        <f>AVERAGEIFS(dataNiveles[Paradas posibles],dataNiveles[Nivel],A4,dataNiveles[Pasos planificados],"&gt;0")</f>
+        <v>8.6904761904761898</v>
+      </c>
+      <c r="V4" cm="1">
+        <f t="array" ref="V4">_xlfn.STDEV.P(IF((dataNiveles[Nivel]=A4)*(dataNiveles[Pasos planificados]&lt;&gt;0),dataNiveles[Paradas posibles]))</f>
+        <v>6.3263925447592557</v>
+      </c>
+      <c r="W4">
+        <f>AVERAGEIFS(dataNiveles[Paradas realizadas],dataNiveles[Nivel],A4,dataNiveles[Pasos planificados],"&gt;0")</f>
+        <v>6.8809523809523814</v>
+      </c>
+      <c r="X4" cm="1">
+        <f t="array" ref="X4">_xlfn.STDEV.P(IF((dataNiveles[Nivel]=A4)*(dataNiveles[Pasos planificados]&lt;&gt;0),dataNiveles[Paradas realizadas]))</f>
+        <v>5.2426927875280933</v>
+      </c>
+      <c r="Y4">
+        <f>AVERAGEIFS(dataNiveles[Errores parada por tiempo excedido],dataNiveles[Nivel],A4,dataNiveles[Pasos planificados],"&gt;0")</f>
+        <v>4.7619047619047616E-2</v>
+      </c>
+      <c r="Z4" cm="1">
+        <f t="array" ref="Z4">_xlfn.STDEV.P(IF((dataNiveles[Nivel]=A4)*(dataNiveles[Pasos planificados]&lt;&gt;0),dataNiveles[Errores parada por tiempo excedido]))</f>
+        <v>0.21295885499997996</v>
+      </c>
+      <c r="AA4">
+        <f>AVERAGEIFS(dataNiveles[Num errores por tiempo excedido],dataNiveles[Nivel],A4,dataNiveles[Pasos planificados],"&gt;0")</f>
+        <v>0.11904761904761904</v>
+      </c>
+      <c r="AB4" cm="1">
+        <f t="array" ref="AB4">_xlfn.STDEV.P(IF((dataNiveles[Nivel]=A4)*(dataNiveles[Pasos planificados]&lt;&gt;0),dataNiveles[Num errores por tiempo excedido]))</f>
+        <v>0.39050522540135058</v>
+      </c>
+      <c r="AC4">
+        <f>AVERAGEIFS(dataNiveles[% Aciertos],dataNiveles[Nivel],A4,dataNiveles[Pasos planificados],"&gt;0")</f>
+        <v>84.838453427840761</v>
+      </c>
+      <c r="AD4" cm="1">
+        <f t="array" ref="AD4">_xlfn.STDEV.P(IF((dataNiveles[Nivel]=A4)*(dataNiveles[Pasos planificados]&lt;&gt;0),dataNiveles[% Aciertos]))</f>
+        <v>12.891775925706845</v>
+      </c>
+      <c r="AE4">
+        <f>AVERAGEIFS(dataNiveles[% Mal],dataNiveles[Nivel],A4,dataNiveles[Pasos planificados],"&gt;0")</f>
+        <v>15.161546572159182</v>
+      </c>
+      <c r="AF4" cm="1">
+        <f t="array" ref="AF4">_xlfn.STDEV.P(IF((dataNiveles[Nivel]=A4)*(dataNiveles[Pasos planificados]&lt;&gt;0),dataNiveles[% Mal]))</f>
+        <v>12.891775925706742</v>
+      </c>
+    </row>
+    <row r="6" spans="1:32" x14ac:dyDescent="0.3">
+      <c r="C6" t="s">
+        <v>335</v>
+      </c>
+      <c r="D6" t="s">
+        <v>336</v>
+      </c>
+      <c r="E6" t="s">
+        <v>337</v>
+      </c>
+      <c r="F6" t="s">
+        <v>338</v>
+      </c>
+      <c r="G6" t="s">
+        <v>347</v>
+      </c>
+      <c r="H6" t="s">
+        <v>349</v>
+      </c>
+      <c r="I6" t="s">
+        <v>348</v>
+      </c>
+      <c r="J6" t="s">
+        <v>350</v>
+      </c>
+    </row>
+    <row r="7" spans="1:32" x14ac:dyDescent="0.3">
+      <c r="C7">
+        <f>AVERAGEIFS(dataNiveles[Tiempo duracion],dataNiveles[Nivel],A2,dataNiveles[Pasos planificados],"&gt;0")</f>
+        <v>745.82640000000004</v>
+      </c>
+      <c r="D7" cm="1">
+        <f t="array" ref="D7">_xlfn.STDEV.P(IF((dataNiveles[Nivel]=A2)*(dataNiveles[Pasos planificados]&lt;&gt;0),dataNiveles[Tiempo duracion]))</f>
+        <v>540.96108448069128</v>
+      </c>
+      <c r="E7">
+        <f>AVERAGEIFS(dataNiveles[Num intentos],dataNiveles[Nivel],A2,dataNiveles[Pasos planificados],"&gt;0")</f>
+        <v>4.1857142857142859</v>
+      </c>
+      <c r="F7" cm="1">
+        <f t="array" ref="F7">_xlfn.STDEV.P(IF((dataNiveles[Nivel]=A2)*(dataNiveles[Pasos planificados]&lt;&gt;0),dataNiveles[Num intentos]))</f>
+        <v>2.9340019336971772</v>
+      </c>
+      <c r="G7">
+        <f>COUNTIFS(dataNiveles[Nivel],A2, dataNiveles[Completado],"VERDADERO",dataNiveles[Pasos planificados],"&gt;0")</f>
+        <v>24</v>
+      </c>
+      <c r="H7">
+        <f>100*G7/B2</f>
+        <v>34.285714285714285</v>
+      </c>
+      <c r="I7">
+        <f>COUNTIFS(dataNiveles[Nivel],A2, dataNiveles[Completado],"FALSO",dataNiveles[Pasos planificados],"&gt;0")</f>
+        <v>46</v>
+      </c>
+      <c r="J7">
+        <f>100*I7/B2</f>
+        <v>65.714285714285708</v>
+      </c>
+    </row>
+    <row r="8" spans="1:32" x14ac:dyDescent="0.3">
+      <c r="C8">
+        <f>AVERAGEIFS(dataNiveles[Tiempo duracion],dataNiveles[Nivel],A3,dataNiveles[Pasos planificados],"&gt;0")</f>
+        <v>678.47790740740754</v>
+      </c>
+      <c r="D8" cm="1">
+        <f t="array" ref="D8">_xlfn.STDEV.P(IF((dataNiveles[Nivel]=A3)*(dataNiveles[Pasos planificados]&lt;&gt;0),dataNiveles[Tiempo duracion]))</f>
+        <v>720.47346805872417</v>
+      </c>
+      <c r="E8">
+        <f>AVERAGEIFS(dataNiveles[Num intentos],dataNiveles[Nivel],A3,dataNiveles[Pasos planificados],"&gt;0")</f>
+        <v>3.074074074074074</v>
+      </c>
+      <c r="F8" cm="1">
+        <f t="array" ref="F8">_xlfn.STDEV.P(IF((dataNiveles[Nivel]=A3)*(dataNiveles[Pasos planificados]&lt;&gt;0),dataNiveles[Num intentos]))</f>
+        <v>3.7998628233127723</v>
+      </c>
+      <c r="G8">
+        <f>COUNTIFS(dataNiveles[Nivel],A3, dataNiveles[Completado],"VERDADERO",dataNiveles[Pasos planificados],"&gt;0")</f>
+        <v>22</v>
+      </c>
+      <c r="H8">
+        <f t="shared" ref="H8:H9" si="0">100*G8/B3</f>
+        <v>40.74074074074074</v>
+      </c>
+      <c r="I8">
+        <f>COUNTIFS(dataNiveles[Nivel],A3, dataNiveles[Completado],"FALSO",dataNiveles[Pasos planificados],"&gt;0")</f>
+        <v>32</v>
+      </c>
+      <c r="J8">
+        <f t="shared" ref="J8:J9" si="1">100*I8/B3</f>
+        <v>59.25925925925926</v>
+      </c>
+    </row>
+    <row r="9" spans="1:32" x14ac:dyDescent="0.3">
+      <c r="C9">
+        <f>AVERAGEIFS(dataNiveles[Tiempo duracion],dataNiveles[Nivel],A4,dataNiveles[Pasos planificados],"&gt;0")</f>
+        <v>501.5519523809524</v>
+      </c>
+      <c r="D9" cm="1">
+        <f t="array" ref="D9">_xlfn.STDEV.P(IF((dataNiveles[Nivel]=A4)*(dataNiveles[Pasos planificados]&lt;&gt;0),dataNiveles[Tiempo duracion]))</f>
+        <v>451.29781997932702</v>
+      </c>
+      <c r="E9">
+        <f>AVERAGEIFS(dataNiveles[Num intentos],dataNiveles[Nivel],A4,dataNiveles[Pasos planificados],"&gt;0")</f>
+        <v>2.7857142857142856</v>
+      </c>
+      <c r="F9" cm="1">
+        <f t="array" ref="F9">_xlfn.STDEV.P(IF((dataNiveles[Nivel]=A4)*(dataNiveles[Pasos planificados]&lt;&gt;0),dataNiveles[Num intentos]))</f>
+        <v>2.0648499805498872</v>
+      </c>
+      <c r="G9">
+        <f>COUNTIFS(dataNiveles[Nivel],A4, dataNiveles[Completado],"VERDADERO",dataNiveles[Pasos planificados],"&gt;0")</f>
+        <v>26</v>
+      </c>
+      <c r="H9">
+        <f t="shared" si="0"/>
+        <v>61.904761904761905</v>
+      </c>
+      <c r="I9">
+        <f>COUNTIFS(dataNiveles[Nivel],A4, dataNiveles[Completado],"FALSO",dataNiveles[Pasos planificados],"&gt;0")</f>
+        <v>16</v>
+      </c>
+      <c r="J9">
+        <f t="shared" si="1"/>
+        <v>38.095238095238095</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Avances análisis de datos
</commit_message>
<xml_diff>
--- a/datosNivelesMedias.xlsx
+++ b/datosNivelesMedias.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\hlocal\C_TFG\Datos\Mision Colombia-20260209T150018Z-3-001\jsonToCsv_TFG\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{91964B7D-C697-43C6-82C1-94F7295EDC54}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ED025CE0-03E4-4F97-8C7A-4BE6BBDF97B6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1138,15 +1138,33 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="3" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.59999389629810485"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.59999389629810485"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -1167,16 +1185,40 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -17334,108 +17376,135 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E7E06012-538D-4879-B4D7-76AF65331837}">
-  <dimension ref="A1:AF9"/>
+  <dimension ref="A1:AN4"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="38" max="38" width="13.5546875" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:32" x14ac:dyDescent="0.3">
-      <c r="A1" t="s">
+    <row r="1" spans="1:40" ht="72" x14ac:dyDescent="0.3">
+      <c r="A1" s="3" t="s">
         <v>307</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="3" t="s">
         <v>308</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="4" t="s">
         <v>309</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="5" t="s">
         <v>310</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="4" t="s">
         <v>311</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="5" t="s">
         <v>312</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="4" t="s">
         <v>313</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="5" t="s">
         <v>314</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="4" t="s">
         <v>315</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="5" t="s">
         <v>316</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="4" t="s">
         <v>317</v>
       </c>
-      <c r="L1" t="s">
+      <c r="L1" s="5" t="s">
         <v>318</v>
       </c>
-      <c r="M1" t="s">
+      <c r="M1" s="4" t="s">
         <v>319</v>
       </c>
-      <c r="N1" t="s">
+      <c r="N1" s="5" t="s">
         <v>320</v>
       </c>
-      <c r="O1" t="s">
+      <c r="O1" s="4" t="s">
         <v>321</v>
       </c>
-      <c r="P1" t="s">
+      <c r="P1" s="5" t="s">
         <v>322</v>
       </c>
-      <c r="Q1" t="s">
+      <c r="Q1" s="4" t="s">
         <v>323</v>
       </c>
-      <c r="R1" t="s">
+      <c r="R1" s="5" t="s">
         <v>324</v>
       </c>
-      <c r="S1" t="s">
+      <c r="S1" s="4" t="s">
         <v>325</v>
       </c>
-      <c r="T1" t="s">
+      <c r="T1" s="5" t="s">
         <v>326</v>
       </c>
-      <c r="U1" t="s">
+      <c r="U1" s="4" t="s">
         <v>327</v>
       </c>
-      <c r="V1" t="s">
+      <c r="V1" s="5" t="s">
         <v>328</v>
       </c>
-      <c r="W1" t="s">
+      <c r="W1" s="4" t="s">
         <v>329</v>
       </c>
-      <c r="X1" t="s">
+      <c r="X1" s="5" t="s">
         <v>330</v>
       </c>
-      <c r="Y1" t="s">
+      <c r="Y1" s="4" t="s">
         <v>331</v>
       </c>
-      <c r="Z1" t="s">
+      <c r="Z1" s="5" t="s">
         <v>332</v>
       </c>
-      <c r="AA1" t="s">
+      <c r="AA1" s="4" t="s">
         <v>333</v>
       </c>
-      <c r="AB1" t="s">
+      <c r="AB1" s="5" t="s">
         <v>334</v>
       </c>
-      <c r="AC1" t="s">
+      <c r="AC1" s="4" t="s">
         <v>343</v>
       </c>
-      <c r="AD1" t="s">
+      <c r="AD1" s="5" t="s">
         <v>344</v>
       </c>
-      <c r="AE1" t="s">
+      <c r="AE1" s="4" t="s">
         <v>345</v>
       </c>
-      <c r="AF1" t="s">
+      <c r="AF1" s="5" t="s">
         <v>346</v>
       </c>
-    </row>
-    <row r="2" spans="1:32" x14ac:dyDescent="0.3">
+      <c r="AG1" s="4" t="s">
+        <v>335</v>
+      </c>
+      <c r="AH1" s="5" t="s">
+        <v>336</v>
+      </c>
+      <c r="AI1" s="4" t="s">
+        <v>337</v>
+      </c>
+      <c r="AJ1" s="5" t="s">
+        <v>338</v>
+      </c>
+      <c r="AK1" s="4" t="s">
+        <v>347</v>
+      </c>
+      <c r="AL1" s="4" t="s">
+        <v>349</v>
+      </c>
+      <c r="AM1" s="4" t="s">
+        <v>348</v>
+      </c>
+      <c r="AN1" s="4" t="s">
+        <v>350</v>
+      </c>
+    </row>
+    <row r="2" spans="1:40" x14ac:dyDescent="0.3">
       <c r="A2">
         <v>1</v>
       </c>
@@ -17563,8 +17632,40 @@
         <f t="array" ref="AF2">_xlfn.STDEV.P(IF((dataNiveles[Nivel]=A2)*(dataNiveles[Pasos planificados]&lt;&gt;0),dataNiveles[% Mal]))</f>
         <v>15.269100509855752</v>
       </c>
-    </row>
-    <row r="3" spans="1:32" x14ac:dyDescent="0.3">
+      <c r="AG2">
+        <f>AVERAGEIFS(dataNiveles[Tiempo duracion],dataNiveles[Nivel],A2,dataNiveles[Pasos planificados],"&gt;0")</f>
+        <v>745.82640000000004</v>
+      </c>
+      <c r="AH2" cm="1">
+        <f t="array" ref="AH2">_xlfn.STDEV.P(IF((dataNiveles[Nivel]=A2)*(dataNiveles[Pasos planificados]&lt;&gt;0),dataNiveles[Tiempo duracion]))</f>
+        <v>540.96108448069128</v>
+      </c>
+      <c r="AI2">
+        <f>AVERAGEIFS(dataNiveles[Num intentos],dataNiveles[Nivel],A2,dataNiveles[Pasos planificados],"&gt;0")</f>
+        <v>4.1857142857142859</v>
+      </c>
+      <c r="AJ2" cm="1">
+        <f t="array" ref="AJ2">_xlfn.STDEV.P(IF((dataNiveles[Nivel]=A2)*(dataNiveles[Pasos planificados]&lt;&gt;0),dataNiveles[Num intentos]))</f>
+        <v>2.9340019336971772</v>
+      </c>
+      <c r="AK2">
+        <f>COUNTIFS(dataNiveles[Nivel],A2, dataNiveles[Completado],"VERDADERO",dataNiveles[Pasos planificados],"&gt;0")</f>
+        <v>24</v>
+      </c>
+      <c r="AL2">
+        <f>100*AK2/B2</f>
+        <v>34.285714285714285</v>
+      </c>
+      <c r="AM2">
+        <f>COUNTIFS(dataNiveles[Nivel],A2, dataNiveles[Completado],"FALSO",dataNiveles[Pasos planificados],"&gt;0")</f>
+        <v>46</v>
+      </c>
+      <c r="AN2">
+        <f>100*AM2/B2</f>
+        <v>65.714285714285708</v>
+      </c>
+    </row>
+    <row r="3" spans="1:40" x14ac:dyDescent="0.3">
       <c r="A3">
         <v>2</v>
       </c>
@@ -17692,8 +17793,40 @@
         <f t="array" ref="AF3">_xlfn.STDEV.P(IF((dataNiveles[Nivel]=A3)*(dataNiveles[Pasos planificados]&lt;&gt;0),dataNiveles[% Mal]))</f>
         <v>21.073686270495212</v>
       </c>
-    </row>
-    <row r="4" spans="1:32" x14ac:dyDescent="0.3">
+      <c r="AG3">
+        <f>AVERAGEIFS(dataNiveles[Tiempo duracion],dataNiveles[Nivel],A3,dataNiveles[Pasos planificados],"&gt;0")</f>
+        <v>678.47790740740754</v>
+      </c>
+      <c r="AH3" cm="1">
+        <f t="array" ref="AH3">_xlfn.STDEV.P(IF((dataNiveles[Nivel]=A3)*(dataNiveles[Pasos planificados]&lt;&gt;0),dataNiveles[Tiempo duracion]))</f>
+        <v>720.47346805872417</v>
+      </c>
+      <c r="AI3">
+        <f>AVERAGEIFS(dataNiveles[Num intentos],dataNiveles[Nivel],A3,dataNiveles[Pasos planificados],"&gt;0")</f>
+        <v>3.074074074074074</v>
+      </c>
+      <c r="AJ3" cm="1">
+        <f t="array" ref="AJ3">_xlfn.STDEV.P(IF((dataNiveles[Nivel]=A3)*(dataNiveles[Pasos planificados]&lt;&gt;0),dataNiveles[Num intentos]))</f>
+        <v>3.7998628233127723</v>
+      </c>
+      <c r="AK3">
+        <f>COUNTIFS(dataNiveles[Nivel],A3, dataNiveles[Completado],"VERDADERO",dataNiveles[Pasos planificados],"&gt;0")</f>
+        <v>22</v>
+      </c>
+      <c r="AL3">
+        <f>100*AK3/B3</f>
+        <v>40.74074074074074</v>
+      </c>
+      <c r="AM3">
+        <f>COUNTIFS(dataNiveles[Nivel],A3, dataNiveles[Completado],"FALSO",dataNiveles[Pasos planificados],"&gt;0")</f>
+        <v>32</v>
+      </c>
+      <c r="AN3">
+        <f>100*AM3/B3</f>
+        <v>59.25925925925926</v>
+      </c>
+    </row>
+    <row r="4" spans="1:40" x14ac:dyDescent="0.3">
       <c r="A4">
         <v>3</v>
       </c>
@@ -17821,132 +17954,36 @@
         <f t="array" ref="AF4">_xlfn.STDEV.P(IF((dataNiveles[Nivel]=A4)*(dataNiveles[Pasos planificados]&lt;&gt;0),dataNiveles[% Mal]))</f>
         <v>12.891775925706742</v>
       </c>
-    </row>
-    <row r="6" spans="1:32" x14ac:dyDescent="0.3">
-      <c r="C6" t="s">
-        <v>335</v>
-      </c>
-      <c r="D6" t="s">
-        <v>336</v>
-      </c>
-      <c r="E6" t="s">
-        <v>337</v>
-      </c>
-      <c r="F6" t="s">
-        <v>338</v>
-      </c>
-      <c r="G6" t="s">
-        <v>347</v>
-      </c>
-      <c r="H6" t="s">
-        <v>349</v>
-      </c>
-      <c r="I6" t="s">
-        <v>348</v>
-      </c>
-      <c r="J6" t="s">
-        <v>350</v>
-      </c>
-    </row>
-    <row r="7" spans="1:32" x14ac:dyDescent="0.3">
-      <c r="C7">
-        <f>AVERAGEIFS(dataNiveles[Tiempo duracion],dataNiveles[Nivel],A2,dataNiveles[Pasos planificados],"&gt;0")</f>
-        <v>745.82640000000004</v>
-      </c>
-      <c r="D7" cm="1">
-        <f t="array" ref="D7">_xlfn.STDEV.P(IF((dataNiveles[Nivel]=A2)*(dataNiveles[Pasos planificados]&lt;&gt;0),dataNiveles[Tiempo duracion]))</f>
-        <v>540.96108448069128</v>
-      </c>
-      <c r="E7">
-        <f>AVERAGEIFS(dataNiveles[Num intentos],dataNiveles[Nivel],A2,dataNiveles[Pasos planificados],"&gt;0")</f>
-        <v>4.1857142857142859</v>
-      </c>
-      <c r="F7" cm="1">
-        <f t="array" ref="F7">_xlfn.STDEV.P(IF((dataNiveles[Nivel]=A2)*(dataNiveles[Pasos planificados]&lt;&gt;0),dataNiveles[Num intentos]))</f>
-        <v>2.9340019336971772</v>
-      </c>
-      <c r="G7">
-        <f>COUNTIFS(dataNiveles[Nivel],A2, dataNiveles[Completado],"VERDADERO",dataNiveles[Pasos planificados],"&gt;0")</f>
-        <v>24</v>
-      </c>
-      <c r="H7">
-        <f>100*G7/B2</f>
-        <v>34.285714285714285</v>
-      </c>
-      <c r="I7">
-        <f>COUNTIFS(dataNiveles[Nivel],A2, dataNiveles[Completado],"FALSO",dataNiveles[Pasos planificados],"&gt;0")</f>
-        <v>46</v>
-      </c>
-      <c r="J7">
-        <f>100*I7/B2</f>
-        <v>65.714285714285708</v>
-      </c>
-    </row>
-    <row r="8" spans="1:32" x14ac:dyDescent="0.3">
-      <c r="C8">
-        <f>AVERAGEIFS(dataNiveles[Tiempo duracion],dataNiveles[Nivel],A3,dataNiveles[Pasos planificados],"&gt;0")</f>
-        <v>678.47790740740754</v>
-      </c>
-      <c r="D8" cm="1">
-        <f t="array" ref="D8">_xlfn.STDEV.P(IF((dataNiveles[Nivel]=A3)*(dataNiveles[Pasos planificados]&lt;&gt;0),dataNiveles[Tiempo duracion]))</f>
-        <v>720.47346805872417</v>
-      </c>
-      <c r="E8">
-        <f>AVERAGEIFS(dataNiveles[Num intentos],dataNiveles[Nivel],A3,dataNiveles[Pasos planificados],"&gt;0")</f>
-        <v>3.074074074074074</v>
-      </c>
-      <c r="F8" cm="1">
-        <f t="array" ref="F8">_xlfn.STDEV.P(IF((dataNiveles[Nivel]=A3)*(dataNiveles[Pasos planificados]&lt;&gt;0),dataNiveles[Num intentos]))</f>
-        <v>3.7998628233127723</v>
-      </c>
-      <c r="G8">
-        <f>COUNTIFS(dataNiveles[Nivel],A3, dataNiveles[Completado],"VERDADERO",dataNiveles[Pasos planificados],"&gt;0")</f>
-        <v>22</v>
-      </c>
-      <c r="H8">
-        <f t="shared" ref="H8:H9" si="0">100*G8/B3</f>
-        <v>40.74074074074074</v>
-      </c>
-      <c r="I8">
-        <f>COUNTIFS(dataNiveles[Nivel],A3, dataNiveles[Completado],"FALSO",dataNiveles[Pasos planificados],"&gt;0")</f>
-        <v>32</v>
-      </c>
-      <c r="J8">
-        <f t="shared" ref="J8:J9" si="1">100*I8/B3</f>
-        <v>59.25925925925926</v>
-      </c>
-    </row>
-    <row r="9" spans="1:32" x14ac:dyDescent="0.3">
-      <c r="C9">
+      <c r="AG4">
         <f>AVERAGEIFS(dataNiveles[Tiempo duracion],dataNiveles[Nivel],A4,dataNiveles[Pasos planificados],"&gt;0")</f>
         <v>501.5519523809524</v>
       </c>
-      <c r="D9" cm="1">
-        <f t="array" ref="D9">_xlfn.STDEV.P(IF((dataNiveles[Nivel]=A4)*(dataNiveles[Pasos planificados]&lt;&gt;0),dataNiveles[Tiempo duracion]))</f>
+      <c r="AH4" cm="1">
+        <f t="array" ref="AH4">_xlfn.STDEV.P(IF((dataNiveles[Nivel]=A4)*(dataNiveles[Pasos planificados]&lt;&gt;0),dataNiveles[Tiempo duracion]))</f>
         <v>451.29781997932702</v>
       </c>
-      <c r="E9">
+      <c r="AI4">
         <f>AVERAGEIFS(dataNiveles[Num intentos],dataNiveles[Nivel],A4,dataNiveles[Pasos planificados],"&gt;0")</f>
         <v>2.7857142857142856</v>
       </c>
-      <c r="F9" cm="1">
-        <f t="array" ref="F9">_xlfn.STDEV.P(IF((dataNiveles[Nivel]=A4)*(dataNiveles[Pasos planificados]&lt;&gt;0),dataNiveles[Num intentos]))</f>
+      <c r="AJ4" cm="1">
+        <f t="array" ref="AJ4">_xlfn.STDEV.P(IF((dataNiveles[Nivel]=A4)*(dataNiveles[Pasos planificados]&lt;&gt;0),dataNiveles[Num intentos]))</f>
         <v>2.0648499805498872</v>
       </c>
-      <c r="G9">
+      <c r="AK4">
         <f>COUNTIFS(dataNiveles[Nivel],A4, dataNiveles[Completado],"VERDADERO",dataNiveles[Pasos planificados],"&gt;0")</f>
         <v>26</v>
       </c>
-      <c r="H9">
-        <f t="shared" si="0"/>
+      <c r="AL4">
+        <f>100*AK4/B4</f>
         <v>61.904761904761905</v>
       </c>
-      <c r="I9">
+      <c r="AM4">
         <f>COUNTIFS(dataNiveles[Nivel],A4, dataNiveles[Completado],"FALSO",dataNiveles[Pasos planificados],"&gt;0")</f>
         <v>16</v>
       </c>
-      <c r="J9">
-        <f t="shared" si="1"/>
+      <c r="AN4">
+        <f>100*AM4/B4</f>
         <v>38.095238095238095</v>
       </c>
     </row>

</xml_diff>